<commit_message>
Orçamentos: aba Vistaprint.ie no comparativo, com produto e configuração por linha
Quarta coluna no comparativo de cotações: o pedido montado no catálogo do
vistaprint.ie (mesh banner 208 × 82 cm personalizado, vinyl banner 100 × 200,
roller banners 85 × 200 e 100 × 200, window lettering e window decal para as
portas, corrugated plastic A2), com a página de cada produto e a configuração a
escolher. Os preços ficam em células de entrada: o site foi recusado pela
política de rede do ambiente e o índice de busca não expõe valores. A coluna
converte o preço exibido para sem IVA e alimenta o comparativo e o resumo.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1FDufm2zVw9d1c3PLPuzV
</commit_message>
<xml_diff>
--- a/Orçamentos/Sinalização/comparativo_cotacoes_2026-09-24.xlsx
+++ b/Orçamentos/Sinalização/comparativo_cotacoes_2026-09-24.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Necessidade" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Banner Printing" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Snap Leeson" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Comparativo" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Vistaprint" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Comparativo" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -67,8 +68,30 @@
 </comments>
 </file>
 
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="I18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Menos 1: a linha de fixação nunca leva preço.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="279">
   <si>
     <t xml:space="preserve">Cotações de sinalização × necessidade do plano — 24/09/2026</t>
   </si>
@@ -85,13 +108,16 @@
     <t xml:space="preserve">Helloprint (ref. 18/09)</t>
   </si>
   <si>
+    <t xml:space="preserve">Vistaprint.ie (a preencher)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nota</t>
   </si>
   <si>
     <t xml:space="preserve">Como foi cotado — subtotal sem IVA</t>
   </si>
   <si>
-    <t xml:space="preserve">Snap: sem a linha Premium (alternativa aos Basic). Helloprint: referência de 18/09, não foi pedido de novo.</t>
+    <t xml:space="preserve">Snap: sem a linha Premium (alternativa aos Basic). Helloprint: referência de 18/09, não foi pedido de novo. Vistaprint: sem cotação formal, é o catálogo online.</t>
   </si>
   <si>
     <t xml:space="preserve">Como foi cotado — total com IVA</t>
@@ -100,7 +126,7 @@
     <t xml:space="preserve">Pedido corrigido — subtotal sem IVA (linhas com preço)</t>
   </si>
   <si>
-    <t xml:space="preserve">Só o que cada gráfica já precificou; ver linhas "a cotar".</t>
+    <t xml:space="preserve">Só o que cada gráfica já precificou; ver linhas "a cotar". Vistaprint fica em zero até a aba dela ser preenchida.</t>
   </si>
   <si>
     <t xml:space="preserve">Pedido corrigido — IVA 23%</t>
@@ -118,7 +144,7 @@
     <t xml:space="preserve">Linhas ainda por cotar</t>
   </si>
   <si>
-    <t xml:space="preserve">Banner Printing: vinil, correx, fixação. Snap: vinil, fixação.</t>
+    <t xml:space="preserve">Banner Printing: vinil, correx, fixação. Snap: vinil, fixação. Vistaprint: as linhas cujo preço ainda não foi colado.</t>
   </si>
   <si>
     <t xml:space="preserve">O que dizer a cada gráfica</t>
@@ -136,6 +162,9 @@
     <t xml:space="preserve">Certo (artefato)</t>
   </si>
   <si>
+    <t xml:space="preserve">Vistaprint.ie</t>
+  </si>
+  <si>
     <t xml:space="preserve">O que corrigir</t>
   </si>
   <si>
@@ -151,6 +180,9 @@
     <t xml:space="preserve">12 (fichas: 11)</t>
   </si>
   <si>
+    <t xml:space="preserve">mesh 208 × 82 cm personalizado</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nada a corrigir no pedido. Internamente: confirmar 12 × 11 antes de fechar.</t>
   </si>
   <si>
@@ -163,6 +195,9 @@
     <t xml:space="preserve">3</t>
   </si>
   <si>
+    <t xml:space="preserve">vinyl banner 100 × 200 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Reduzir de 12 para 3. As 12 foram copiadas do número de fence banners.</t>
   </si>
   <si>
@@ -175,6 +210,9 @@
     <t xml:space="preserve">1 × € 333</t>
   </si>
   <si>
+    <t xml:space="preserve">roller banner 100 × 200 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Snap: subir de 1 para 3. Banner Printing está certo.</t>
   </si>
   <si>
@@ -190,6 +228,9 @@
     <t xml:space="preserve">16</t>
   </si>
   <si>
+    <t xml:space="preserve">roller banner 85 × 200 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nada a corrigir. Snap: escolher Basic ou Premium.</t>
   </si>
   <si>
@@ -205,6 +246,9 @@
     <t xml:space="preserve">4</t>
   </si>
   <si>
+    <t xml:space="preserve">3 × window lettering (≤ 50 × 50 cm) + 1 × window decal (S7)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Banner Printing: trocar o banner 90 × 90 por vinil adesivo recortado (letras A/B/C de 300 mm + pictogramas da S7), removível. Snap: pedir a linha.</t>
   </si>
   <si>
@@ -217,6 +261,9 @@
     <t xml:space="preserve">2</t>
   </si>
   <si>
+    <t xml:space="preserve">corrugated plastic A2, 3,5 ou 5 mm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Banner Printing: pedir a linha. Snap está certo (5 mm serve).</t>
   </si>
   <si>
@@ -226,6 +273,9 @@
     <t xml:space="preserve">verba ~€ 40</t>
   </si>
   <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
     <t xml:space="preserve">Não é item de gráfica; comprar à parte.</t>
   </si>
   <si>
@@ -238,7 +288,7 @@
     <t xml:space="preserve">não informado</t>
   </si>
   <si>
-    <t xml:space="preserve">—</t>
+    <t xml:space="preserve">no checkout (economy / standard / fast)</t>
   </si>
   <si>
     <t xml:space="preserve">Snap: perguntar frete ou retirada. Prazo: eleição em 04/10.</t>
@@ -262,7 +312,10 @@
     <t xml:space="preserve">5. Cores e fonte: rolo azul #33507E, amarelo #E8C63A, vermelho #C8102E (proposta até o rolo chegar), Montserrat. Pedir prova de cor antes de imprimir a tiragem.</t>
   </si>
   <si>
-    <t xml:space="preserve">Legenda: azul = número digitado das cotações/artefato · amarelo = quantidade a corrigir · vermelho = linha não cotada · verde = linha certa. Preços em EUR, IVA irlandês 23%.</t>
+    <t xml:space="preserve">6. Vistaprint.ie (24/09): o produto e a configuração de cada linha estão na aba Vistaprint, mas o site foi bloqueado pela política de rede do ambiente e o índice de busca não expõe preços. As células amarelas da aba recebem o preço do configurador; o comparativo e este resumo se atualizam sozinhos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legenda: azul = número digitado das cotações/artefato · amarelo = a preencher ou quantidade a corrigir · vermelho = linha não cotada · verde = linha certa · verde-escuro = link para outra aba. Preços em EUR, IVA irlandês 23%.</t>
   </si>
   <si>
     <t xml:space="preserve">O que o plano de sinalização precisa (artefato "Plano de Sinalização · Posto de Dublin", rev. 23/09/2026)</t>
@@ -646,10 +699,163 @@
     <t xml:space="preserve">A proposta diz "print-ready PDF with crop marks and bleed": arte final é por nossa conta.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pedido corrigido — os três preços lado a lado (sem IVA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quantidades: aba Necessidade. Helloprint IE = cotação de referência de 18/09 usada no artefato (catálogo online). Unitários em azul; vazio = não cotado.</t>
+    <t xml:space="preserve">Vistaprint.ie — pedido montado no catálogo, preços a preencher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produto e configuração conferidos no índice de busca do vistaprint.ie em 24/09/2026; o site em si está bloqueado pela rede deste ambiente, então o preço de cada linha fica em amarelo, para colar do configurador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linha do plano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produto Vistaprint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuração a escolher no site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Página</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preço unit. como o site mostra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inclui IVA? (S/N)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit. sem IVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total sem IVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mesh banner (custom size)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho personalizado 208 × 82 cm · poliéster 190 gsm sem PVC (uso repetido, até 2 anos) ou 115 gsm (uso curto) · ilhoses metálicos de 1,3 cm a cada 60 cm, contados automaticamente no tamanho personalizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.vistaprint.ie/signs-posters/banners/mesh-banners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os tamanhos de catálogo vão de 50 × 100 a 100 × 300 cm; 208 × 82 é personalizado (máximo 300 × 1200 cm). Mesh deixa o vento passar, como o Declan recomendou.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinyl banner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho de catálogo 100 × 200 cm · 10 ilhoses · 1 face</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.vistaprint.ie/signs-posters/banners/vinyl-banners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parede leste do Hall 2 (P2), abrigada do vento: vinil sólido serve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinil recortado por porta (A, B, C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Window lettering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho personalizado (o site aceita de 15 × 5 até 50 × 50 cm) · uma letra de 300 mm por porta · sem fundo visível · material UV, à prova d'água, sem PVC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.vistaprint.ie/labels-stickers/stickers/window-lettering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O plano prevê 1200 × 700 mm por porta, mas o conteúdo é uma letra de 300 mm: cabe num lettering de 40 × 40 cm. Conferir com o Posto se a peça é só a letra. Remoção sem resíduo: confirmar na página do produto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinil da porta preferencial S7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Window decal (opaco, removível)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho personalizado ~120 × 30 cm para os cinco pictogramas de 200 mm (ou 2 peças de 60 × 30) · opaco · aplicação por dentro do vidro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.vistaprint.ie/signs-posters/window-decals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O lettering para em 50 × 50 cm, por isso a S7 vai em window decal. Tamanho máximo do decal: conferir no configurador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roller banner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho 100 × 200 cm · cassete, haste, banner e bolsa incluídos · uso interno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.vistaprint.ie/signs-posters/banners/roller-banners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painéis das portas A, B e C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho 85 × 200 cm · cassete, haste, banner e bolsa incluídos · uso interno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As 16 placas de grupo. Conferir se há desconto por quantidade no configurador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrugated plastic sign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A2 (42 × 59,4 cm) · 3,5 mm ou 5 mm · 1 face</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.vistaprint.ie/signs-posters/plastic-signs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saídas S2 e S8. O plano diz 4 mm; o site oferece 3,5 e 5 mm — 5 mm é o mais próximo do correx da Snap.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não é item da Vistaprint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verba de ~€ 40; tie wraps, ganchos magnéticos e fita compram-se à parte.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Economy / Standard / Fast, escolhido no checkout; produção em 1–2 dias úteis, pedido antes das 21h CET entra no mesmo dia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.vistaprint.ie/delivery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eleição em 04/10: escolher a velocidade que chega até 01/10 e anotar aqui o valor do frete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal sem IVA (linhas preenchidas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alíquota de IVA (Irlanda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linhas ainda sem preço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como preencher: abra cada página, monte o produto com a configuração da coluna C e a quantidade da coluna E, e cole em F o preço unitário que o site mostrar. Em G, diga se o valor exibido já inclui IVA (S) ou não (N): a coluna H converte para sem IVA e o comparativo usa H.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O que já se sabe do catálogo (índice de busca, 24/09): mesh em 190 ou 115 gsm com ilhoses a cada 60 cm e personalizado até 300 × 1200 cm; vinyl banner 100 × 200 cm com 10 ilhoses; roller banner em 85 × 200 e 100 × 200 com cassete, haste e bolsa; corrugated plastic em 3,5 e 5 mm; window lettering personalizado até 50 × 50 cm; window decals em transparente ou opaco, removíveis. Nenhum preço aparece no índice: só o configurador mostra.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloqueio: www.vistaprint.ie, vistaprint.co.uk e web.archive.org foram recusados pela política de rede do ambiente em que esta planilha foi montada. Liberar o domínio nas configurações do ambiente permite preencher a coluna F automaticamente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedido corrigido — os quatro preços lado a lado (sem IVA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantidades: aba Necessidade. Helloprint IE = referência de 18/09 usada no artefato. Vistaprint = aba Vistaprint (preços a preencher). Unitários em azul; vazio = não cotado.</t>
   </si>
   <si>
     <t xml:space="preserve">Modelo</t>
@@ -673,13 +879,19 @@
     <t xml:space="preserve">Snap Leeson total</t>
   </si>
   <si>
-    <t xml:space="preserve">Helloprint: unitário do artefato. Snap: € 1.320 / 12.</t>
+    <t xml:space="preserve">Vistaprint unit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vistaprint total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: unitário do artefato. Snap: € 1.320 / 12. Vistaprint: mesh 208 × 82 cm personalizado.</t>
   </si>
   <si>
     <t xml:space="preserve">Helloprint: premissa do artefato (não precificada). Snap: € 1.320 / 12, premissa para 3 un.</t>
   </si>
   <si>
-    <t xml:space="preserve">Premissa do artefato; nenhuma das duas gráficas cotou o item certo.</t>
+    <t xml:space="preserve">Premissa do artefato; nenhuma das duas gráficas cotou o item certo. Vistaprint: 3 window lettering + 1 window decal, média das 4 peças.</t>
   </si>
   <si>
     <t xml:space="preserve">Helloprint: € 92,58 / 3 (deduzido do total de 18/09). Snap: cotou 1 un.; premissa para 3.</t>
@@ -688,13 +900,13 @@
     <t xml:space="preserve">Helloprint: € 397,99 / 16 (deduzido do total de 18/09). Snap "Basic"; a "Premium" sai a € 154,69/un.</t>
   </si>
   <si>
-    <t xml:space="preserve">Premissa do artefato; Banner Printing não cotou; Snap: corriboard 5 mm.</t>
+    <t xml:space="preserve">Premissa do artefato; Banner Printing não cotou; Snap: corriboard 5 mm; Vistaprint: 3,5 ou 5 mm.</t>
   </si>
   <si>
     <t xml:space="preserve">Verba; compra à parte.</t>
   </si>
   <si>
-    <t xml:space="preserve">Helloprint: Saver grátis (28/09). Banner Printing: € 15. Snap: não informou.</t>
+    <t xml:space="preserve">Helloprint: Saver grátis (28/09). Banner Printing: € 15. Snap: não informou. Vistaprint: frete do checkout, aba Vistaprint.</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal sem IVA (linhas com preço)</t>
@@ -710,6 +922,9 @@
   </si>
   <si>
     <t xml:space="preserve">Helloprint IE: preços de catálogo de 18/09, quatro linhas são premissa (PVC, vinil, correx, fixação) e o prazo Saver (28/09) já passou do upload de 18/09 13:30 — para entregar antes de 04/10 seria preciso reconferir prazos e frete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vistaprint: a coluna vem da aba Vistaprint e fica vazia até os preços serem colados lá. O unitário do vinil é a média das quatro peças (3 lettering + 1 decal), para caber na linha única do plano.</t>
   </si>
   <si>
     <t xml:space="preserve">Sensibilidade: se o número certo de fence banners for 11 e não 12, tire um unitário de fence banner de cada coluna (Helloprint € 32,40; Banner Printing € 70; Snap € 110, sem IVA).</t>
@@ -727,7 +942,7 @@
     <numFmt numFmtId="168" formatCode="0%"/>
     <numFmt numFmtId="169" formatCode="0.0\×"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -819,6 +1034,21 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -835,14 +1065,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2E6E4"/>
-        <bgColor rgb="FFD9EAD3"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFE2E6E4"/>
+        <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -907,7 +1137,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -936,11 +1166,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -948,11 +1186,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -972,11 +1214,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1000,7 +1242,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1024,7 +1266,39 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1036,7 +1310,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1077,7 +1351,7 @@
       <rgbColor rgb="FFE2E6E4"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0563C1"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -1296,12 +1570,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1312,6 +1586,7 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -1321,6 +1596,7 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
@@ -1328,6 +1604,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4"/>
@@ -1343,10 +1620,13 @@
       <c r="E4" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F4" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="6" t="n">
         <f aca="false">'Banner Printing'!D13</f>
@@ -1357,13 +1637,14 @@
         <v>4453</v>
       </c>
       <c r="D5" s="6"/>
-      <c r="E5" s="7" t="s">
-        <v>7</v>
+      <c r="E5" s="7"/>
+      <c r="F5" s="8" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">'Banner Printing'!D15</f>
@@ -1375,30 +1656,35 @@
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="7"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="9" t="n">
+      <c r="F6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="10" t="n">
         <f aca="false">'Banner Printing'!G13</f>
         <v>3108</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <f aca="false">'Snap Leeson'!G13</f>
         <v>4129</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10" t="n">
         <f aca="false">Comparativo!D13</f>
         <v>1234.37</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>10</v>
+      <c r="E7" s="11" t="n">
+        <f aca="false">Comparativo!J13</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">'Banner Printing'!G14</f>
@@ -1412,29 +1698,37 @@
         <f aca="false">Comparativo!D14</f>
         <v>283.9051</v>
       </c>
-      <c r="E8" s="7"/>
+      <c r="E8" s="7" t="n">
+        <f aca="false">Comparativo!J14</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="9" t="n">
+      <c r="A9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="10" t="n">
         <f aca="false">'Banner Printing'!G15</f>
         <v>3822.84</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="10" t="n">
         <f aca="false">'Snap Leeson'!G15</f>
         <v>5078.67</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="10" t="n">
         <f aca="false">Comparativo!D15</f>
         <v>1518.2751</v>
       </c>
-      <c r="E9" s="10"/>
+      <c r="E9" s="11" t="n">
+        <f aca="false">Comparativo!J15</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">'Banner Printing'!H13</f>
@@ -1445,27 +1739,32 @@
         <v>-324</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="E10" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E10" s="7"/>
+      <c r="F10" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="B11" s="13" t="n">
         <f aca="false">COUNTIF('Banner Printing'!G5:G12,"a cotar")</f>
         <v>3</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="13" t="n">
         <f aca="false">COUNTIF('Snap Leeson'!G5:G12,"a cotar")</f>
         <v>2</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>16</v>
+      <c r="E11" s="14" t="n">
+        <f aca="false">Comparativo!J16</f>
+        <v>8</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1474,167 +1773,196 @@
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>17</v>
+      <c r="A13" s="15" t="s">
+        <v>18</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="F14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="7" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="B15" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>27</v>
       </c>
+      <c r="D15" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E16" s="7" t="s">
+      <c r="A16" s="8" t="s">
         <v>31</v>
       </c>
+      <c r="B16" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="7" t="s">
+      <c r="A17" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>35</v>
+      <c r="E17" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="A18" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B18" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E18" s="8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+      <c r="F18" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="7" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="B19" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>49</v>
       </c>
+      <c r="D19" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>57</v>
+      <c r="A21" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1643,85 +1971,105 @@
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="s">
-        <v>58</v>
+      <c r="A24" s="15" t="s">
+        <v>67</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
+      <c r="A25" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
     </row>
     <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
+      <c r="A27" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
+      <c r="A28" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
     </row>
     <row r="29" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="A29" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+    </row>
+    <row r="30" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A31:E31"/>
+  <mergeCells count="7">
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A32:F32"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1751,7 +2099,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1761,7 +2109,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1779,436 +2127,436 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E5" s="15" t="n">
+      <c r="A5" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>77</v>
+      <c r="F5" s="8" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="15" t="n">
+      <c r="A6" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>79</v>
+      <c r="F6" s="8" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="15" t="n">
+      <c r="A7" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>82</v>
+      <c r="F7" s="8" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="A8" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="7" t="s">
-        <v>89</v>
+      <c r="F9" s="8" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E10" s="15" t="n">
+      <c r="A10" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>92</v>
+      <c r="F10" s="8" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E11" s="15" t="n">
+      <c r="A11" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="7" t="s">
-        <v>94</v>
+      <c r="F11" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E12" s="15" t="n">
+      <c r="A12" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E12" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>94</v>
+      <c r="F12" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="15" t="n">
+      <c r="A13" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="7" t="s">
-        <v>97</v>
+      <c r="F13" s="8" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E14" s="15" t="n">
+      <c r="A14" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E14" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>100</v>
+      <c r="F14" s="8" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E15" s="15" t="n">
+      <c r="A15" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E15" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E16" s="15" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E17" s="15" t="n">
+      <c r="F17" s="8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E18" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E18" s="15" t="n">
+      <c r="F18" s="8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E19" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E19" s="15" t="n">
+      <c r="F19" s="8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E20" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E20" s="15" t="n">
+      <c r="F20" s="8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E21" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E21" s="15" t="n">
+      <c r="F21" s="8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E24" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="E22" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="E23" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>124</v>
+      <c r="F24" s="8" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8" t="n">
+      <c r="A25" s="9"/>
+      <c r="B25" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9" t="n">
         <f aca="false">SUM(E5:E24)</f>
         <v>40</v>
       </c>
-      <c r="F25" s="8"/>
+      <c r="F25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
@@ -2219,8 +2567,8 @@
       <c r="F26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
-        <v>126</v>
+      <c r="A27" s="15" t="s">
+        <v>136</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -2230,22 +2578,22 @@
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2253,21 +2601,21 @@
         <v>1</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C29" s="16" t="n">
+        <v>85</v>
+      </c>
+      <c r="C29" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D29" s="20" t="n">
         <f aca="false">SUMIF($C$5:$C$24,B29,$E$5:$E$24)</f>
         <v>11</v>
       </c>
-      <c r="E29" s="17" t="n">
+      <c r="E29" s="20" t="n">
         <f aca="false">C29-D29</f>
         <v>1</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>132</v>
+      <c r="F29" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2275,9 +2623,9 @@
         <v>2</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="C30" s="21" t="n">
         <v>3</v>
       </c>
       <c r="D30" s="5" t="n">
@@ -2288,16 +2636,16 @@
         <f aca="false">C30-D30</f>
         <v>0</v>
       </c>
-      <c r="F30" s="7"/>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C31" s="18" t="n">
+        <v>112</v>
+      </c>
+      <c r="C31" s="21" t="n">
         <v>4</v>
       </c>
       <c r="D31" s="5" t="n">
@@ -2308,8 +2656,8 @@
         <f aca="false">C31-D31</f>
         <v>0</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>133</v>
+      <c r="F31" s="8" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2317,9 +2665,9 @@
         <v>4</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="18" t="n">
+        <v>36</v>
+      </c>
+      <c r="C32" s="21" t="n">
         <v>3</v>
       </c>
       <c r="D32" s="5" t="n">
@@ -2330,16 +2678,16 @@
         <f aca="false">C32-D32</f>
         <v>0</v>
       </c>
-      <c r="F32" s="7"/>
+      <c r="F32" s="8"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="n">
         <v>5</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C33" s="18" t="n">
+        <v>41</v>
+      </c>
+      <c r="C33" s="21" t="n">
         <v>16</v>
       </c>
       <c r="D33" s="5" t="n">
@@ -2350,16 +2698,16 @@
         <f aca="false">C33-D33</f>
         <v>0</v>
       </c>
-      <c r="F33" s="7"/>
+      <c r="F33" s="8"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="n">
         <v>6</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="C34" s="18" t="n">
+        <v>130</v>
+      </c>
+      <c r="C34" s="21" t="n">
         <v>2</v>
       </c>
       <c r="D34" s="5" t="n">
@@ -2370,8 +2718,8 @@
         <f aca="false">C34-D34</f>
         <v>0</v>
       </c>
-      <c r="F34" s="7" t="s">
-        <v>134</v>
+      <c r="F34" s="8" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2379,9 +2727,9 @@
         <v>7</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C35" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="C35" s="21" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="5" t="n">
@@ -2392,28 +2740,28 @@
         <f aca="false">C35-D35</f>
         <v>0</v>
       </c>
-      <c r="F35" s="7" t="s">
-        <v>135</v>
+      <c r="F35" s="8" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="8"/>
-      <c r="B36" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="C36" s="8" t="n">
+      <c r="A36" s="9"/>
+      <c r="B36" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="C36" s="9" t="n">
         <f aca="false">SUM(C29:C35)</f>
         <v>41</v>
       </c>
-      <c r="D36" s="8" t="n">
+      <c r="D36" s="9" t="n">
         <f aca="false">SUM(D29:D35)</f>
         <v>40</v>
       </c>
-      <c r="E36" s="8" t="n">
+      <c r="E36" s="9" t="n">
         <f aca="false">SUM(E29:E35)</f>
         <v>1</v>
       </c>
-      <c r="F36" s="8"/>
+      <c r="F36" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2448,7 +2796,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2461,7 +2809,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2485,51 +2833,51 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>131</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="B5" s="20" t="n">
+      <c r="A5" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="B5" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="24" t="n">
         <v>70</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">B5*C5</f>
         <v>840</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="F5" s="22" t="n">
+      <c r="E5" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="F5" s="25" t="n">
         <v>12</v>
       </c>
       <c r="G5" s="6" t="n">
@@ -2540,28 +2888,28 @@
         <f aca="false">IF(ISNUMBER(G5),G5-D5,-D5)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="7" t="s">
-        <v>147</v>
+      <c r="I5" s="8" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="B6" s="16" t="n">
+      <c r="A6" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="B6" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="24" t="n">
         <v>74</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">B6*C6</f>
         <v>888</v>
       </c>
-      <c r="E6" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="17" t="n">
+      <c r="E6" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="20" t="n">
         <v>3</v>
       </c>
       <c r="G6" s="6" t="n">
@@ -2572,28 +2920,28 @@
         <f aca="false">IF(ISNUMBER(G6),G6-D6,-D6)</f>
         <v>-666</v>
       </c>
-      <c r="I6" s="7" t="s">
-        <v>149</v>
+      <c r="I6" s="8" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="B7" s="20" t="n">
+      <c r="A7" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B7" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="24" t="n">
         <v>149</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">B7*C7</f>
         <v>447</v>
       </c>
-      <c r="E7" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="22" t="n">
+      <c r="E7" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="25" t="n">
         <v>3</v>
       </c>
       <c r="G7" s="6" t="n">
@@ -2604,28 +2952,28 @@
         <f aca="false">IF(ISNUMBER(G7),G7-D7,-D7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>151</v>
+      <c r="I7" s="8" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
-        <v>152</v>
-      </c>
-      <c r="B8" s="20" t="n">
+      <c r="A8" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>16</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="24" t="n">
         <v>99</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">B8*C8</f>
         <v>1584</v>
       </c>
-      <c r="E8" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="F8" s="22" t="n">
+      <c r="E8" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="25" t="n">
         <v>16</v>
       </c>
       <c r="G8" s="6" t="n">
@@ -2636,29 +2984,29 @@
         <f aca="false">IF(ISNUMBER(G8),G8-D8,-D8)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>153</v>
+      <c r="I8" s="8" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="B9" s="16" t="n">
+      <c r="A9" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="24" t="n">
         <v>35</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">B9*C9</f>
         <v>140</v>
       </c>
-      <c r="E9" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>156</v>
+      <c r="E9" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>166</v>
       </c>
       <c r="G9" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F9),F9*C9,"a cotar")</f>
@@ -2668,26 +3016,26 @@
         <f aca="false">IF(ISNUMBER(G9),G9-D9,-D9)</f>
         <v>-140</v>
       </c>
-      <c r="I9" s="7" t="s">
-        <v>157</v>
+      <c r="I9" s="8" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" s="18" t="n">
+      <c r="A10" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="24" t="n">
         <v>15</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">B10*C10</f>
         <v>15</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>53</v>
+      <c r="E10" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>1</v>
@@ -2700,131 +3048,131 @@
         <f aca="false">IF(ISNUMBER(G10),G10-D10,-D10)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>159</v>
+      <c r="I10" s="8" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
-        <v>160</v>
-      </c>
-      <c r="B11" s="25" t="n">
+      <c r="A11" s="27" t="s">
+        <v>170</v>
+      </c>
+      <c r="B11" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="26" t="s">
-        <v>120</v>
-      </c>
-      <c r="F11" s="26" t="n">
+      <c r="E11" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="H11" s="28" t="s">
-        <v>156</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>161</v>
+      <c r="G11" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="H11" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="B12" s="25" t="n">
+      <c r="A12" s="27" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="F12" s="26" t="n">
+      <c r="E12" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="F12" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="H12" s="28" t="s">
-        <v>156</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>163</v>
+      <c r="G12" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="H12" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9" t="n">
+      <c r="A13" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10" t="n">
         <f aca="false">SUM(D5:D12)</f>
         <v>3914</v>
       </c>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="9" t="n">
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="10" t="n">
         <f aca="false">SUM(G5:G10)</f>
         <v>3108</v>
       </c>
-      <c r="H13" s="9" t="n">
+      <c r="H13" s="10" t="n">
         <f aca="false">G13-D13</f>
         <v>-806</v>
       </c>
-      <c r="I13" s="8"/>
+      <c r="I13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="B14" s="29" t="n">
+      <c r="A14" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B14" s="32" t="n">
         <v>0.23</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9" t="n">
+      <c r="C14" s="9"/>
+      <c r="D14" s="10" t="n">
         <f aca="false">D13*$B$14</f>
         <v>900.22</v>
       </c>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="9" t="n">
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="10" t="n">
         <f aca="false">G13*$B$14</f>
         <v>714.84</v>
       </c>
-      <c r="H14" s="9" t="n">
+      <c r="H14" s="10" t="n">
         <f aca="false">G14-D14</f>
         <v>-185.38</v>
       </c>
-      <c r="I14" s="8"/>
+      <c r="I14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9" t="n">
+      <c r="A15" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="10" t="n">
         <f aca="false">D13+D14</f>
         <v>4814.22</v>
       </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="9" t="n">
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="10" t="n">
         <f aca="false">G13+G14</f>
         <v>3822.84</v>
       </c>
-      <c r="H15" s="9" t="n">
+      <c r="H15" s="10" t="n">
         <f aca="false">G15-D15</f>
         <v>-991.38</v>
       </c>
-      <c r="I15" s="8"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
@@ -2839,7 +3187,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -2852,7 +3200,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -2865,7 +3213,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -2908,7 +3256,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2921,7 +3269,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2945,51 +3293,51 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>131</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
-        <v>172</v>
-      </c>
-      <c r="B5" s="20" t="n">
+      <c r="A5" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="B5" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="24" t="n">
         <v>110</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">B5*C5</f>
         <v>1320</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="F5" s="22" t="n">
+      <c r="E5" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="F5" s="25" t="n">
         <v>12</v>
       </c>
       <c r="G5" s="6" t="n">
@@ -3000,28 +3348,28 @@
         <f aca="false">IF(ISNUMBER(G5),G5-D5,-D5)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="7" t="s">
-        <v>173</v>
+      <c r="I5" s="8" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>174</v>
-      </c>
-      <c r="B6" s="16" t="n">
+      <c r="A6" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="24" t="n">
         <v>110</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">B6*C6</f>
         <v>1320</v>
       </c>
-      <c r="E6" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="17" t="n">
+      <c r="E6" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="20" t="n">
         <v>3</v>
       </c>
       <c r="G6" s="6" t="n">
@@ -3032,28 +3380,28 @@
         <f aca="false">IF(ISNUMBER(G6),G6-D6,-D6)</f>
         <v>-990</v>
       </c>
-      <c r="I6" s="7" t="s">
-        <v>175</v>
+      <c r="I6" s="8" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="B7" s="16" t="n">
+      <c r="A7" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="24" t="n">
         <v>333</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">B7*C7</f>
         <v>333</v>
       </c>
-      <c r="E7" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="17" t="n">
+      <c r="E7" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="20" t="n">
         <v>3</v>
       </c>
       <c r="G7" s="6" t="n">
@@ -3064,28 +3412,28 @@
         <f aca="false">IF(ISNUMBER(G7),G7-D7,-D7)</f>
         <v>666</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>177</v>
+      <c r="I7" s="8" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
-        <v>178</v>
-      </c>
-      <c r="B8" s="20" t="n">
+      <c r="A8" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>16</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="24" t="n">
         <v>90</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">B8*C8</f>
         <v>1440</v>
       </c>
-      <c r="E8" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="F8" s="22" t="n">
+      <c r="E8" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="25" t="n">
         <v>16</v>
       </c>
       <c r="G8" s="6" t="n">
@@ -3096,26 +3444,26 @@
         <f aca="false">IF(ISNUMBER(G8),G8-D8,-D8)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>179</v>
+      <c r="I8" s="8" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="B9" s="18" t="n">
+      <c r="A9" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="B9" s="21" t="n">
         <v>16</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="24" t="n">
         <v>154.6875</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">B9*C9</f>
         <v>2475</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>181</v>
+      <c r="E9" s="8" t="s">
+        <v>191</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>0</v>
@@ -3123,31 +3471,31 @@
       <c r="G9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>183</v>
+      <c r="H9" s="31" t="s">
+        <v>192</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
-        <v>184</v>
-      </c>
-      <c r="B10" s="20" t="n">
+      <c r="A10" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="B10" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">B10*C10</f>
         <v>40</v>
       </c>
-      <c r="E10" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="F10" s="22" t="n">
+      <c r="E10" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="F10" s="25" t="n">
         <v>2</v>
       </c>
       <c r="G10" s="6" t="n">
@@ -3158,131 +3506,131 @@
         <f aca="false">IF(ISNUMBER(G10),G10-D10,-D10)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>185</v>
+      <c r="I10" s="8" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
-        <v>186</v>
-      </c>
-      <c r="B11" s="25" t="n">
+      <c r="A11" s="27" t="s">
+        <v>196</v>
+      </c>
+      <c r="B11" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="F11" s="26" t="n">
+      <c r="E11" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="F11" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="H11" s="28" t="s">
-        <v>156</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>187</v>
+      <c r="G11" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="H11" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="B12" s="25" t="n">
+      <c r="A12" s="27" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="F12" s="26" t="n">
+      <c r="E12" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="F12" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="H12" s="28" t="s">
-        <v>156</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>188</v>
+      <c r="G12" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="H12" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9" t="n">
+      <c r="A13" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10" t="n">
         <f aca="false">SUM(D5:D12)-D9</f>
         <v>4453</v>
       </c>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="9" t="n">
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="10" t="n">
         <f aca="false">SUM(G5:G10)</f>
         <v>4129</v>
       </c>
-      <c r="H13" s="9" t="n">
+      <c r="H13" s="10" t="n">
         <f aca="false">G13-D13</f>
         <v>-324</v>
       </c>
-      <c r="I13" s="8"/>
+      <c r="I13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="B14" s="29" t="n">
+      <c r="A14" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B14" s="32" t="n">
         <v>0.23</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9" t="n">
+      <c r="C14" s="9"/>
+      <c r="D14" s="10" t="n">
         <f aca="false">D13*$B$14</f>
         <v>1024.19</v>
       </c>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="9" t="n">
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="10" t="n">
         <f aca="false">G13*$B$14</f>
         <v>949.67</v>
       </c>
-      <c r="H14" s="9" t="n">
+      <c r="H14" s="10" t="n">
         <f aca="false">G14-D14</f>
         <v>-74.52</v>
       </c>
-      <c r="I14" s="8"/>
+      <c r="I14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9" t="n">
+      <c r="A15" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="10" t="n">
         <f aca="false">D13+D14</f>
         <v>5477.19</v>
       </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="9" t="n">
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="10" t="n">
         <f aca="false">G13+G14</f>
         <v>5078.67</v>
       </c>
-      <c r="H15" s="9" t="n">
+      <c r="H15" s="10" t="n">
         <f aca="false">G15-D15</f>
         <v>-398.52</v>
       </c>
-      <c r="I15" s="8"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
@@ -3297,7 +3645,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -3310,7 +3658,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -3323,7 +3671,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3351,20 +3699,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3374,10 +3725,11 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3387,6 +3739,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
@@ -3398,395 +3751,1028 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>71</v>
+        <v>205</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>197</v>
+        <v>81</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>211</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="D5" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <f aca="false">Necessidade!$C$29</f>
+        <v>12</v>
+      </c>
+      <c r="F5" s="34"/>
+      <c r="G5" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H5" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(F5),IF(UPPER(G5)="S",F5/(1+$B$17),F5),"")</f>
+        <v/>
+      </c>
+      <c r="I5" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(H5),E5*H5,"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="D6" s="33" t="s">
+        <v>219</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <f aca="false">Necessidade!$C$30</f>
+        <v>3</v>
+      </c>
+      <c r="F6" s="34"/>
+      <c r="G6" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H6" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(F6),IF(UPPER(G6)="S",F6/(1+$B$17),F6),"")</f>
+        <v/>
+      </c>
+      <c r="I6" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(H6),E6*H6,"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="D7" s="33" t="s">
+        <v>224</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="34"/>
+      <c r="G7" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H7" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(F7),IF(UPPER(G7)="S",F7/(1+$B$17),F7),"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(H7),E7*H7,"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="D8" s="33" t="s">
+        <v>229</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="34"/>
+      <c r="G8" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H8" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(F8),IF(UPPER(G8)="S",F8/(1+$B$17),F8),"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(H8),E8*H8,"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="D9" s="33" t="s">
+        <v>233</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <f aca="false">Necessidade!$C$32</f>
+        <v>3</v>
+      </c>
+      <c r="F9" s="34"/>
+      <c r="G9" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H9" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(F9),IF(UPPER(G9)="S",F9/(1+$B$17),F9),"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(H9),E9*H9,"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="D10" s="33" t="s">
+        <v>233</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <f aca="false">Necessidade!$C$33</f>
+        <v>16</v>
+      </c>
+      <c r="F10" s="34"/>
+      <c r="G10" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H10" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(F10),IF(UPPER(G10)="S",F10/(1+$B$17),F10),"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(H10),E10*H10,"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="D11" s="33" t="s">
+        <v>239</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <f aca="false">Necessidade!$C$34</f>
+        <v>2</v>
+      </c>
+      <c r="F11" s="34"/>
+      <c r="G11" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H11" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(F11),IF(UPPER(G11)="S",F11/(1+$B$17),F11),"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(H11),E11*H11,"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5" t="n">
+        <f aca="false">Necessidade!$C$35</f>
+        <v>1</v>
+      </c>
+      <c r="F12" s="24"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="D13" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="34"/>
+      <c r="G13" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H13" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(F13),IF(UPPER(G13)="S",F13/(1+$B$17),F13),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="6" t="str">
+        <f aca="false">IF(ISNUMBER(H13),E13*H13,"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="10" t="n">
+        <f aca="false">SUM(I5:I13)</f>
+        <v>0</v>
+      </c>
+      <c r="J14" s="9"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="10" t="n">
+        <f aca="false">I14*$B$17</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="9"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="10" t="n">
+        <f aca="false">I14+I15</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="37" t="s">
+        <v>248</v>
+      </c>
+      <c r="B17" s="38" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="37"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="37" t="s">
+        <v>249</v>
+      </c>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37" t="n">
+        <f aca="false">COUNTBLANK(F5:F13)-1</f>
+        <v>8</v>
+      </c>
+      <c r="J18" s="37"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="B20" s="39"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="39"/>
+      <c r="I20" s="39"/>
+      <c r="J20" s="39"/>
+    </row>
+    <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="39" t="s">
+        <v>251</v>
+      </c>
+      <c r="B21" s="39"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="39"/>
+      <c r="I21" s="39"/>
+      <c r="J21" s="39"/>
+    </row>
+    <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39" t="s">
+        <v>252</v>
+      </c>
+      <c r="B22" s="39"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="39"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="39"/>
+      <c r="I22" s="39"/>
+      <c r="J22" s="39"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A22:J22"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="D5" r:id="rId2" display="https://www.vistaprint.ie/signs-posters/banners/mesh-banners"/>
+    <hyperlink ref="D6" r:id="rId3" display="https://www.vistaprint.ie/signs-posters/banners/vinyl-banners"/>
+    <hyperlink ref="D7" r:id="rId4" display="https://www.vistaprint.ie/labels-stickers/stickers/window-lettering"/>
+    <hyperlink ref="D8" r:id="rId5" display="https://www.vistaprint.ie/signs-posters/window-decals"/>
+    <hyperlink ref="D9" r:id="rId6" display="https://www.vistaprint.ie/signs-posters/banners/roller-banners"/>
+    <hyperlink ref="D10" r:id="rId7" display="https://www.vistaprint.ie/signs-posters/banners/roller-banners"/>
+    <hyperlink ref="D11" r:id="rId8" display="https://www.vistaprint.ie/signs-posters/plastic-signs"/>
+    <hyperlink ref="D13" r:id="rId9" display="https://www.vistaprint.ie/delivery"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId10"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">Necessidade!$C$29</f>
         <v>12</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="24" t="n">
         <v>32.4</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C5),$B5*C5,"")</f>
         <v>388.8</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="24" t="n">
         <v>70</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E5),$B5*E5,"")</f>
         <v>840</v>
       </c>
-      <c r="G5" s="21" t="n">
+      <c r="G5" s="24" t="n">
         <v>110</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G5),$B5*G5,"")</f>
         <v>1320</v>
       </c>
-      <c r="I5" s="7" t="s">
-        <v>201</v>
+      <c r="I5" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(Vistaprint!$H$5),Vistaprint!$H$5,"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="7" t="str">
+        <f aca="false">IF(ISNUMBER(I5),$B5*I5,"")</f>
+        <v/>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">Necessidade!$C$30</f>
         <v>3</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="24" t="n">
         <v>55</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C6),$B6*C6,"")</f>
         <v>165</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="24" t="n">
         <v>74</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E6),$B6*E6,"")</f>
         <v>222</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="24" t="n">
         <v>110</v>
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G6),$B6*G6,"")</f>
         <v>330</v>
       </c>
-      <c r="I6" s="7" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I6" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(Vistaprint!$H$6),Vistaprint!$H$6,"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="7" t="str">
+        <f aca="false">IF(ISNUMBER(I6),$B6*I6,"")</f>
+        <v/>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">Necessidade!$C$31</f>
         <v>4</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="24" t="n">
         <v>30</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C7),$B7*C7,"")</f>
         <v>120</v>
       </c>
-      <c r="E7" s="30"/>
-      <c r="F7" s="31" t="str">
+      <c r="E7" s="41"/>
+      <c r="F7" s="42" t="str">
         <f aca="false">IF(ISNUMBER(E7),$B7*E7,"")</f>
         <v/>
       </c>
-      <c r="G7" s="30"/>
-      <c r="H7" s="31" t="str">
+      <c r="G7" s="41"/>
+      <c r="H7" s="42" t="str">
         <f aca="false">IF(ISNUMBER(G7),$B7*G7,"")</f>
         <v/>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>203</v>
+      <c r="I7" s="40" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Vistaprint!$H$7),ISNUMBER(Vistaprint!$H$8)),(Vistaprint!$I$7+Vistaprint!$I$8)/(Vistaprint!$E$7+Vistaprint!$E$8),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="7" t="str">
+        <f aca="false">IF(ISNUMBER(I7),$B7*I7,"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">Necessidade!$C$32</f>
         <v>3</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="24" t="n">
         <v>30.86</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C8),$B8*C8,"")</f>
         <v>92.58</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="24" t="n">
         <v>149</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E8),$B8*E8,"")</f>
         <v>447</v>
       </c>
-      <c r="G8" s="21" t="n">
+      <c r="G8" s="24" t="n">
         <v>333</v>
       </c>
       <c r="H8" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G8),$B8*G8,"")</f>
         <v>999</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>204</v>
+      <c r="I8" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(Vistaprint!$H$9),Vistaprint!$H$9,"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="7" t="str">
+        <f aca="false">IF(ISNUMBER(I8),$B8*I8,"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">Necessidade!$C$33</f>
         <v>16</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="24" t="n">
         <v>24.874375</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C9),$B9*C9,"")</f>
         <v>397.99</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="24" t="n">
         <v>99</v>
       </c>
       <c r="F9" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E9),$B9*E9,"")</f>
         <v>1584</v>
       </c>
-      <c r="G9" s="21" t="n">
+      <c r="G9" s="24" t="n">
         <v>90</v>
       </c>
       <c r="H9" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G9),$B9*G9,"")</f>
         <v>1440</v>
       </c>
-      <c r="I9" s="7" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I9" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(Vistaprint!$H$10),Vistaprint!$H$10,"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="7" t="str">
+        <f aca="false">IF(ISNUMBER(I9),$B9*I9,"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Necessidade!$C$34</f>
         <v>2</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="24" t="n">
         <v>15</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C10),$B10*C10,"")</f>
         <v>30</v>
       </c>
-      <c r="E10" s="30"/>
-      <c r="F10" s="31" t="str">
+      <c r="E10" s="41"/>
+      <c r="F10" s="42" t="str">
         <f aca="false">IF(ISNUMBER(E10),$B10*E10,"")</f>
         <v/>
       </c>
-      <c r="G10" s="21" t="n">
+      <c r="G10" s="24" t="n">
         <v>20</v>
       </c>
       <c r="H10" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G10),$B10*G10,"")</f>
         <v>40</v>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>206</v>
+      <c r="I10" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(Vistaprint!$H$11),Vistaprint!$H$11,"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="7" t="str">
+        <f aca="false">IF(ISNUMBER(I10),$B10*I10,"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">Necessidade!$C$35</f>
         <v>1</v>
       </c>
-      <c r="C11" s="21" t="n">
+      <c r="C11" s="24" t="n">
         <v>40</v>
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C11),$B11*C11,"")</f>
         <v>40</v>
       </c>
-      <c r="E11" s="30"/>
-      <c r="F11" s="31" t="str">
+      <c r="E11" s="41"/>
+      <c r="F11" s="42" t="str">
         <f aca="false">IF(ISNUMBER(E11),$B11*E11,"")</f>
         <v/>
       </c>
-      <c r="G11" s="30"/>
-      <c r="H11" s="31" t="str">
+      <c r="G11" s="41"/>
+      <c r="H11" s="42" t="str">
         <f aca="false">IF(ISNUMBER(G11),$B11*G11,"")</f>
         <v/>
       </c>
-      <c r="I11" s="7" t="s">
-        <v>207</v>
+      <c r="I11" s="43"/>
+      <c r="J11" s="42" t="str">
+        <f aca="false">IF(ISNUMBER(I11),$B11*I11,"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C12),$B12*C12,"")</f>
         <v>0</v>
       </c>
-      <c r="E12" s="21" t="n">
+      <c r="E12" s="24" t="n">
         <v>15</v>
       </c>
       <c r="F12" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E12),$B12*E12,"")</f>
         <v>15</v>
       </c>
-      <c r="G12" s="30"/>
-      <c r="H12" s="31" t="str">
+      <c r="G12" s="41"/>
+      <c r="H12" s="42" t="str">
         <f aca="false">IF(ISNUMBER(G12),$B12*G12,"")</f>
         <v/>
       </c>
-      <c r="I12" s="5" t="s">
-        <v>208</v>
+      <c r="I12" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(Vistaprint!$H$13),Vistaprint!$H$13,"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="7" t="str">
+        <f aca="false">IF(ISNUMBER(I12),$B12*I12,"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9" t="n">
+      <c r="A13" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10" t="n">
         <f aca="false">SUM(D5:D12)</f>
         <v>1234.37</v>
       </c>
-      <c r="E13" s="8"/>
-      <c r="F13" s="9" t="n">
+      <c r="E13" s="9"/>
+      <c r="F13" s="10" t="n">
         <f aca="false">SUM(F5:F12)</f>
         <v>3108</v>
       </c>
-      <c r="G13" s="8"/>
-      <c r="H13" s="9" t="n">
+      <c r="G13" s="9"/>
+      <c r="H13" s="10" t="n">
         <f aca="false">SUM(H5:H12)</f>
         <v>4129</v>
       </c>
-      <c r="I13" s="8"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="10" t="n">
+        <f aca="false">SUM(J5:J12)</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="B14" s="29" t="n">
+      <c r="A14" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B14" s="32" t="n">
         <v>0.23</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9" t="n">
+      <c r="C14" s="9"/>
+      <c r="D14" s="10" t="n">
         <f aca="false">D13*$B$14</f>
         <v>283.9051</v>
       </c>
-      <c r="E14" s="8"/>
-      <c r="F14" s="9" t="n">
+      <c r="E14" s="9"/>
+      <c r="F14" s="10" t="n">
         <f aca="false">F13*$B$14</f>
         <v>714.84</v>
       </c>
-      <c r="G14" s="8"/>
-      <c r="H14" s="9" t="n">
+      <c r="G14" s="9"/>
+      <c r="H14" s="10" t="n">
         <f aca="false">H13*$B$14</f>
         <v>949.67</v>
       </c>
-      <c r="I14" s="8"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="10" t="n">
+        <f aca="false">J13*$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9" t="n">
+      <c r="A15" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="10" t="n">
         <f aca="false">D13+D14</f>
         <v>1518.2751</v>
       </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="9" t="n">
+      <c r="E15" s="9"/>
+      <c r="F15" s="10" t="n">
         <f aca="false">F13+F14</f>
         <v>3822.84</v>
       </c>
-      <c r="G15" s="8"/>
-      <c r="H15" s="9" t="n">
+      <c r="G15" s="9"/>
+      <c r="H15" s="10" t="n">
         <f aca="false">H13+H14</f>
         <v>5078.67</v>
       </c>
-      <c r="I15" s="8"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="10" t="n">
+        <f aca="false">J13+J14</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32" t="s">
-        <v>210</v>
-      </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32" t="n">
+      <c r="A16" s="37" t="s">
+        <v>273</v>
+      </c>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37" t="n">
         <f aca="false">COUNTBLANK(C5:C12)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32" t="n">
+      <c r="E16" s="37"/>
+      <c r="F16" s="37" t="n">
         <f aca="false">COUNTBLANK(E5:E12)</f>
         <v>3</v>
       </c>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32" t="n">
+      <c r="G16" s="37"/>
+      <c r="H16" s="37" t="n">
         <f aca="false">COUNTBLANK(G5:G12)</f>
         <v>3</v>
       </c>
-      <c r="I16" s="32"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="37" t="n">
+        <f aca="false">COUNTBLANK(I5:I12)</f>
+        <v>8</v>
+      </c>
+      <c r="K16" s="37"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32" t="s">
-        <v>211</v>
-      </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="33" t="n">
+      <c r="A17" s="37" t="s">
+        <v>274</v>
+      </c>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="44" t="n">
         <f aca="false">IFERROR(F13/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(E5:E12)),"")</f>
         <v>2.97595679692063</v>
       </c>
-      <c r="G17" s="32"/>
-      <c r="H17" s="33" t="n">
+      <c r="G17" s="37"/>
+      <c r="H17" s="44" t="n">
         <f aca="false">IFERROR(H13/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(G5:G12)),"")</f>
         <v>3.84318251626535</v>
       </c>
-      <c r="I17" s="32"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="44" t="str">
+        <f aca="false">IFERROR(J13/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(I5:I12)),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="37"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
@@ -3798,10 +4784,12 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>212</v>
+        <v>275</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3811,10 +4799,12 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>213</v>
+        <v>276</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -3824,10 +4814,12 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>214</v>
+        <v>277</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -3837,6 +4829,23 @@
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Orçamentos: carrinho Helloprint de 24/09 substitui a referência de 18/09 no comparativo
Aba nova com as 33 linhas do carrinho (3 roller banners Medium, 16 Small, 12
fence banners RPET 208 × 82, 3 mesh 200 × 82, 2 window stickers 42 × 60), o
desconto de € 123 e o frete grátis: € 3.314,46 com IVA, € 2.694,68 sem. A
coluna Helloprint do comparativo e do resumo passa a ler dali. A referência de
18/09 (€ 1.234,37) fica registrada como superada: supunha preço de tiragem para
peças de arte diferente, e no carrinho cada arte é uma linha de 1.

Duas leituras do carrinho ficam marcadas como premissa: os 3 mesh 200 × 82 como
a lateral leste (P2) e os 2 stickers 42 × 60 como as saídas (P7). Faltam no
carrinho os 4 vinis das portas e a fixação.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1FDufm2zVw9d1c3PLPuzV
</commit_message>
<xml_diff>
--- a/Orçamentos/Sinalização/comparativo_cotacoes_2026-09-24.xlsx
+++ b/Orçamentos/Sinalização/comparativo_cotacoes_2026-09-24.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Necessidade" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Banner Printing" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Snap Leeson" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Vistaprint" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Comparativo" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Helloprint 24-09" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Vistaprint" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Comparativo" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -68,7 +69,7 @@
 </comments>
 </file>
 
-<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
     <author>Unknown Author</author>
@@ -91,12 +92,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="321">
   <si>
     <t xml:space="preserve">Cotações de sinalização × necessidade do plano — 24/09/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Eleições 2026 · Posto de Dublin · RDS Hall 2. Duas cotações recebidas em 24/09 contra as 40 peças (+ fixação) do artefato de 23/09.</t>
+    <t xml:space="preserve">Eleições 2026 · Posto de Dublin · RDS Hall 2. Duas cotações recebidas e um carrinho Helloprint montado em 24/09, contra as 40 peças (+ fixação) do artefato de 23/09; Vistaprint a preencher.</t>
   </si>
   <si>
     <t xml:space="preserve">Banner Printing (e-mail)</t>
@@ -105,7 +106,7 @@
     <t xml:space="preserve">Snap Leeson (ref. 1554129)</t>
   </si>
   <si>
-    <t xml:space="preserve">Helloprint (ref. 18/09)</t>
+    <t xml:space="preserve">Helloprint (carrinho 24/09)</t>
   </si>
   <si>
     <t xml:space="preserve">Vistaprint.ie (a preencher)</t>
@@ -117,7 +118,7 @@
     <t xml:space="preserve">Como foi cotado — subtotal sem IVA</t>
   </si>
   <si>
-    <t xml:space="preserve">Snap: sem a linha Premium (alternativa aos Basic). Helloprint: referência de 18/09, não foi pedido de novo. Vistaprint: sem cotação formal, é o catálogo online.</t>
+    <t xml:space="preserve">Snap: sem a linha Premium (alternativa aos Basic). Helloprint: carrinho de 24/09 com o desconto de € 100 e frete grátis. Vistaprint: sem cotação formal, é o catálogo online.</t>
   </si>
   <si>
     <t xml:space="preserve">Como foi cotado — total com IVA</t>
@@ -126,7 +127,7 @@
     <t xml:space="preserve">Pedido corrigido — subtotal sem IVA (linhas com preço)</t>
   </si>
   <si>
-    <t xml:space="preserve">Só o que cada gráfica já precificou; ver linhas "a cotar". Vistaprint fica em zero até a aba dela ser preenchida.</t>
+    <t xml:space="preserve">Só o que cada gráfica já precificou; ver linhas "a cotar". Helloprint: igual ao carrinho, porque o carrinho já é o pedido — o que falta nele (4 vinis, fixação) falta aqui também. Vistaprint fica em zero até a aba dela ser preenchida.</t>
   </si>
   <si>
     <t xml:space="preserve">Pedido corrigido — IVA 23%</t>
@@ -144,7 +145,7 @@
     <t xml:space="preserve">Linhas ainda por cotar</t>
   </si>
   <si>
-    <t xml:space="preserve">Banner Printing: vinil, correx, fixação. Snap: vinil, fixação. Vistaprint: as linhas cujo preço ainda não foi colado.</t>
+    <t xml:space="preserve">Banner Printing: vinil, correx, fixação. Snap: vinil, fixação. Helloprint: vinil, fixação. Vistaprint: as linhas cujo preço ainda não foi colado.</t>
   </si>
   <si>
     <t xml:space="preserve">O que dizer a cada gráfica</t>
@@ -159,6 +160,9 @@
     <t xml:space="preserve">Snap Leeson</t>
   </si>
   <si>
+    <t xml:space="preserve">Helloprint carrinho 24/09</t>
+  </si>
+  <si>
     <t xml:space="preserve">Certo (artefato)</t>
   </si>
   <si>
@@ -177,13 +181,16 @@
     <t xml:space="preserve">12 × € 110 (lote € 1.320)</t>
   </si>
   <si>
+    <t xml:space="preserve">12 × € 93,47 c/ IVA (RPET 208 × 82, linhas de 1)</t>
+  </si>
+  <si>
     <t xml:space="preserve">12 (fichas: 11)</t>
   </si>
   <si>
     <t xml:space="preserve">mesh 208 × 82 cm personalizado</t>
   </si>
   <si>
-    <t xml:space="preserve">Nada a corrigir no pedido. Internamente: confirmar 12 × 11 antes de fechar.</t>
+    <t xml:space="preserve">Nada a corrigir no pedido. Internamente: confirmar 12 × 11 antes de fechar. Helloprint: RPET, não mesh — conferir se serve no gradil.</t>
   </si>
   <si>
     <t xml:space="preserve">Banner PVC 2000 × 1000 mm</t>
@@ -192,13 +199,16 @@
     <t xml:space="preserve">12 × € 74</t>
   </si>
   <si>
+    <t xml:space="preserve">3 × mesh 200 × 82 (linha de € 128,74 c/ IVA) — premissa: é a P2?</t>
+  </si>
+  <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
     <t xml:space="preserve">vinyl banner 100 × 200 cm</t>
   </si>
   <si>
-    <t xml:space="preserve">Reduzir de 12 para 3. As 12 foram copiadas do número de fence banners.</t>
+    <t xml:space="preserve">Reduzir de 12 para 3. As 12 foram copiadas do número de fence banners. Helloprint: se os 3 mesh forem a P2, a arte (2:1) precisa ser refeita para 200 × 82.</t>
   </si>
   <si>
     <t xml:space="preserve">Pull-up 1000 × 2000 mm</t>
@@ -210,10 +220,13 @@
     <t xml:space="preserve">1 × € 333</t>
   </si>
   <si>
+    <t xml:space="preserve">3 × € 146,36 c/ IVA (Medium)</t>
+  </si>
+  <si>
     <t xml:space="preserve">roller banner 100 × 200 cm</t>
   </si>
   <si>
-    <t xml:space="preserve">Snap: subir de 1 para 3. Banner Printing está certo.</t>
+    <t xml:space="preserve">Snap: subir de 1 para 3. Banner Printing e Helloprint estão certos.</t>
   </si>
   <si>
     <t xml:space="preserve">Pull-up 850 × 2000 mm</t>
@@ -225,6 +238,9 @@
     <t xml:space="preserve">16 × € 90 (Basic) ou € 154,69 (Premium)</t>
   </si>
   <si>
+    <t xml:space="preserve">16 × € 104,54 c/ IVA (Small)</t>
+  </si>
+  <si>
     <t xml:space="preserve">16</t>
   </si>
   <si>
@@ -243,13 +259,16 @@
     <t xml:space="preserve">não cotado</t>
   </si>
   <si>
+    <t xml:space="preserve">não está no carrinho</t>
+  </si>
+  <si>
     <t xml:space="preserve">4</t>
   </si>
   <si>
     <t xml:space="preserve">3 × window lettering (≤ 50 × 50 cm) + 1 × window decal (S7)</t>
   </si>
   <si>
-    <t xml:space="preserve">Banner Printing: trocar o banner 90 × 90 por vinil adesivo recortado (letras A/B/C de 300 mm + pictogramas da S7), removível. Snap: pedir a linha.</t>
+    <t xml:space="preserve">Banner Printing: trocar o banner 90 × 90 por vinil adesivo recortado (letras A/B/C de 300 mm + pictogramas da S7), removível. Snap: pedir a linha. Helloprint: acrescentar ao carrinho.</t>
   </si>
   <si>
     <t xml:space="preserve">Placa correx 4 mm A2 (594 × 420)</t>
@@ -258,13 +277,16 @@
     <t xml:space="preserve">2 × € 20 (corriboard 5 mm)</t>
   </si>
   <si>
+    <t xml:space="preserve">2 × window sticker 42 × 60 (linha de € 75,36 c/ IVA) — premissa: são as saídas?</t>
+  </si>
+  <si>
     <t xml:space="preserve">2</t>
   </si>
   <si>
     <t xml:space="preserve">corrugated plastic A2, 3,5 ou 5 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Banner Printing: pedir a linha. Snap está certo (5 mm serve).</t>
+    <t xml:space="preserve">Banner Printing: pedir a linha. Snap está certo (5 mm serve). Helloprint: adesivo no batente em vez de placa — decisão do Posto.</t>
   </si>
   <si>
     <t xml:space="preserve">Fixação (tie wraps, ímãs, fita)</t>
@@ -288,10 +310,13 @@
     <t xml:space="preserve">não informado</t>
   </si>
   <si>
+    <t xml:space="preserve">grátis, Standard até 30/09; desconto de € 123 c/ IVA no carrinho</t>
+  </si>
+  <si>
     <t xml:space="preserve">no checkout (economy / standard / fast)</t>
   </si>
   <si>
-    <t xml:space="preserve">Snap: perguntar frete ou retirada. Prazo: eleição em 04/10.</t>
+    <t xml:space="preserve">Snap: perguntar frete ou retirada. Prazo: eleição em 04/10. Helloprint: pedir até 21h de 24/09 para manter as datas.</t>
   </si>
   <si>
     <t xml:space="preserve">Ressalvas</t>
@@ -306,7 +331,7 @@
     <t xml:space="preserve">3. Os dois totais corrigidos não incluem o vinil recortado nem a fixação; o da Banner Printing também não inclui as placas correx. Comparar só depois de as gráficas cotarem o que falta.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Ambas as gráficas ficam bem acima da referência de 18/09 do Helloprint (ver aba Comparativo, linha "Múltiplo"). O Helloprint, porém, era catálogo online com prazo já vencido e quatro linhas sem preço.</t>
+    <t xml:space="preserve">4. O carrinho Helloprint de 24/09 (€ 2.694,68 sem IVA, € 3.314,46 com IVA, já com € 100 de desconto) superou a referência de 18/09 (€ 1.234,37): aquela supunha preço de tiragem para peças de arte diferente. Ainda assim fica abaixo da Banner Printing e da Snap nas linhas comparáveis (aba Comparativo, linha "Múltiplo"). Falta nele o vinil das quatro portas, e duas linhas são premissa de leitura: os 3 mesh 200 × 82 como P2 e os 2 stickers 42 × 60 como saídas.</t>
   </si>
   <si>
     <t xml:space="preserve">5. Cores e fonte: rolo azul #33507E, amarelo #E8C63A, vermelho #C8102E (proposta até o rolo chegar), Montserrat. Pedir prova de cor antes de imprimir a tiragem.</t>
@@ -699,6 +724,111 @@
     <t xml:space="preserve">A proposta diz "print-ready PDF with crop marks and bleed": arte final é por nossa conta.</t>
   </si>
   <si>
+    <t xml:space="preserve">Helloprint IE — carrinho montado em 24/09/2026 (18:59), preços com IVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fonte: PDF "Your Cart" (helloprint.com/en-ie/cart), 12 páginas. Cada peça entrou como linha própria de quantidade 1, porque cada uma tem arte diferente; por isso não há desconto de tiragem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item no carrinho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuração</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linhas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qtd por linha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit. com IVA (site)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit. sem IVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total sem IVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corresponde a (plano)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roller Banners — Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 × 200 cm · Silver budget stand · Basic base · Standard PVC · Standard delivery by Wed 30 Sept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painéis das portas A, B e C. Três linhas de 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roller Banners — Small</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85 × 200 cm · Silver budget stand · Basic base · Standard PVC · Standard delivery by Wed 30 Sept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As 16 placas de grupo. Dezesseis linhas de 1: a referência de 18/09 (€ 24,87/un) supunha 15 iguais numa linha só, o que não existe — cada placa tem arte própria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard Fence Banners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">208 × 82 cm · Recycled RPET Material · Rings every 30 cm, with hems · Banner only · Standard delivery by Tue 29 Sept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doze linhas de 1. RPET (110 gsm) e não o mesh: conferir opacidade e vento. Mesmo ponto da referência de 18/09: € 32,40/un supunha 10 iguais.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banners — Windproof Perforated Mesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 × 82 cm · 1 m² · Rings every 30 cm, with hems · Without Elastic Bands · Express delivery by Tue 29 Sept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREMISSA: lido como a lateral leste (P2), que o plano prevê em 2000 × 1000 mm PVC. Em 200 × 82 a arte da P2 (1000 × 500 px, 2:1) não cabe sem refazer. Linha de 3 a € 128,74.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Window stickers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rectangle or Square · 0,5 m² · White · 42 × 60 cm · Express delivery by Tue 29 Sept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREMISSA: lido como as saídas S2 e S8 (P7, A2 = 42 × 59,4 cm), em adesivo branco no lugar do correx. Linha de 2 a € 75,36. Se for outra coisa, corrigir aqui.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produtos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desconto aplicado no carrinho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O carrinho anuncia € 100 de desconto e abate € 123,00 com IVA (= € 100 sem IVA). Conferir se vale no checkout.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grátis. Entrega Standard até 30/09 (roller banners), 29/09 (fence banners); stickers e mesh em Express, 29/09. Pedido até 21h de 24/09 para essas datas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IVA (Irlanda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O carrinho informa IVA incluído de € 619,83; a conta linha a linha dá € 619,78 (arredondamento de centavos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conferência: 3 × 146,36 + 16 × 104,54 + 12 × 93,47 + 128,74 + 75,36 = € 3.437,46, igual ao "Products incl. VAT" do carrinho; menos € 123,00 = € 3.314,46, igual ao "Total incl. VAT".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O que o carrinho não tem: os 4 vinis recortados das portas (A, B, C e S7) e a fixação. O que ele tem de diferente do plano: a lateral leste em mesh 200 × 82 (não PVC 200 × 100) e as saídas em adesivo 42 × 60 (não correx A2) — as duas leituras acima são premissa desta planilha, não do carrinho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por que subiu contra a referência de 18/09 (€ 1.234,37 sem IVA): aquela conta usou o preço por tiragem (10 fence banners iguais, 15 roller banners iguais) para peças que têm arte diferente. No carrinho cada arte é uma linha de 1, e o unitário é o de 1. As peças que se repetem — P0-Consulta ×2 e P0-Mestra ×2 — poderiam ir em duas linhas de 2 e ter o preço de 2; o resto não.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vistaprint.ie — pedido montado no catálogo, preços a preencher</t>
   </si>
   <si>
@@ -723,12 +853,6 @@
     <t xml:space="preserve">Inclui IVA? (S/N)</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit. sem IVA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total sem IVA</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mesh banner (custom size)</t>
   </si>
   <si>
@@ -822,9 +946,6 @@
     <t xml:space="preserve">Verba de ~€ 40; tie wraps, ganchos magnéticos e fita compram-se à parte.</t>
   </si>
   <si>
-    <t xml:space="preserve">Frete</t>
-  </si>
-  <si>
     <t xml:space="preserve">Economy / Standard / Fast, escolhido no checkout; produção em 1–2 dias úteis, pedido antes das 21h CET entra no mesmo dia</t>
   </si>
   <si>
@@ -855,16 +976,16 @@
     <t xml:space="preserve">Pedido corrigido — os quatro preços lado a lado (sem IVA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantidades: aba Necessidade. Helloprint IE = referência de 18/09 usada no artefato. Vistaprint = aba Vistaprint (preços a preencher). Unitários em azul; vazio = não cotado.</t>
+    <t xml:space="preserve">Quantidades: aba Necessidade. Helloprint = carrinho de 24/09 (aba Helloprint 24-09), sem IVA. Vistaprint = aba Vistaprint (preços a preencher). Unitários em azul; verde-escuro = link de outra aba; vazio = não cotado.</t>
   </si>
   <si>
     <t xml:space="preserve">Modelo</t>
   </si>
   <si>
-    <t xml:space="preserve">Helloprint unit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helloprint total</t>
+    <t xml:space="preserve">Helloprint 24/09 unit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint 24/09 total</t>
   </si>
   <si>
     <t xml:space="preserve">Banner Printing unit.</t>
@@ -885,28 +1006,34 @@
     <t xml:space="preserve">Vistaprint total</t>
   </si>
   <si>
-    <t xml:space="preserve">Helloprint: unitário do artefato. Snap: € 1.320 / 12. Vistaprint: mesh 208 × 82 cm personalizado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helloprint: premissa do artefato (não precificada). Snap: € 1.320 / 12, premissa para 3 un.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Premissa do artefato; nenhuma das duas gráficas cotou o item certo. Vistaprint: 3 window lettering + 1 window decal, média das 4 peças.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helloprint: € 92,58 / 3 (deduzido do total de 18/09). Snap: cotou 1 un.; premissa para 3.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helloprint: € 397,99 / 16 (deduzido do total de 18/09). Snap "Basic"; a "Premium" sai a € 154,69/un.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Premissa do artefato; Banner Printing não cotou; Snap: corriboard 5 mm; Vistaprint: 3,5 ou 5 mm.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verba; compra à parte.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helloprint: Saver grátis (28/09). Banner Printing: € 15. Snap: não informou. Vistaprint: frete do checkout, aba Vistaprint.</t>
+    <t xml:space="preserve">Helloprint: RPET 208 × 82, 12 linhas de 1 (€ 93,47 c/ IVA). Snap: € 1.320 / 12. Vistaprint: mesh 208 × 82 cm personalizado. Ref. 18/09: € 32,40.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: PREMISSA — os 3 mesh 200 × 82 do carrinho lidos como a P2 (formato diferente). Snap: € 1.320 / 12, premissa para 3 un. Ref. 18/09: € 55.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não está no carrinho nem foi cotado pelas duas gráficas. Vistaprint: 3 window lettering + 1 window decal, média das 4 peças. Ref. 18/09: € 30 (premissa).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: Medium, 3 linhas de 1 (€ 146,36 c/ IVA). Snap: cotou 1 un.; premissa para 3. Ref. 18/09: € 30,86.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: Small, 16 linhas de 1 (€ 104,54 c/ IVA). Snap "Basic"; a "Premium" sai a € 154,69/un. Ref. 18/09: € 24,87.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: PREMISSA — os 2 window stickers 42 × 60 do carrinho lidos como as saídas. Snap: corriboard 5 mm; Vistaprint: 3,5 ou 5 mm. Ref. 18/09: € 15.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verba de ~€ 40; compra à parte, ninguém cota.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: grátis (Standard até 30/09). Banner Printing: € 15. Snap: não informou. Vistaprint: frete do checkout, aba Vistaprint.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desconto do carrinho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: € 100 sem IVA (€ 123 com IVA) aplicado no carrinho; ninguém mais ofereceu desconto. Fica fora da linha "Múltiplo".</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal sem IVA (linhas com preço)</t>
@@ -915,19 +1042,19 @@
     <t xml:space="preserve">Linhas sem preço nesta coluna</t>
   </si>
   <si>
-    <t xml:space="preserve">Múltiplo sobre o Helloprint (só linhas com preço)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leitura: os subtotais não são comparáveis linha a linha porque cada coluna cobre um conjunto diferente de itens. A linha "Múltiplo" compara cada gráfica com o Helloprint só nos itens que ela precificou.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helloprint IE: preços de catálogo de 18/09, quatro linhas são premissa (PVC, vinil, correx, fixação) e o prazo Saver (28/09) já passou do upload de 18/09 13:30 — para entregar antes de 04/10 seria preciso reconferir prazos e frete.</t>
+    <t xml:space="preserve">Múltiplo sobre o Helloprint 24/09 (só linhas que os dois precificaram, sem o desconto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leitura: os subtotais não são comparáveis linha a linha porque cada coluna cobre um conjunto diferente de itens. A linha "Múltiplo" compara cada gráfica com o carrinho Helloprint só nos itens que os dois precificaram, e ignora o desconto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: a coluna é o carrinho de 24/09 (aba Helloprint 24-09), com IVA retirado. A referência de 18/09 do artefato (€ 1.234,37 sem IVA) foi superada: supunha preço de tiragem para peças de arte diferente. Duas linhas do carrinho são premissa desta leitura: os 3 mesh 200 × 82 como P2 e os 2 stickers 42 × 60 como saídas.</t>
   </si>
   <si>
     <t xml:space="preserve">Vistaprint: a coluna vem da aba Vistaprint e fica vazia até os preços serem colados lá. O unitário do vinil é a média das quatro peças (3 lettering + 1 decal), para caber na linha única do plano.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sensibilidade: se o número certo de fence banners for 11 e não 12, tire um unitário de fence banner de cada coluna (Helloprint € 32,40; Banner Printing € 70; Snap € 110, sem IVA).</t>
+    <t xml:space="preserve">Sensibilidade: se o número certo de fence banners for 11 e não 12, tire um unitário de fence banner de cada coluna (Helloprint € 75,99; Banner Printing € 70; Snap € 110, sem IVA).</t>
   </si>
 </sst>
 </file>
@@ -1137,7 +1264,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1202,6 +1329,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1242,10 +1373,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1270,6 +1397,26 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1286,23 +1433,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1310,7 +1449,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1570,12 +1709,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1587,6 +1726,7 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -1597,6 +1737,7 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
@@ -1605,6 +1746,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4"/>
@@ -1623,8 +1765,9 @@
       <c r="F4" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
@@ -1636,11 +1779,15 @@
         <f aca="false">'Snap Leeson'!D13</f>
         <v>4453</v>
       </c>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6" t="n">
+        <f aca="false">'Helloprint 24-09'!H13</f>
+        <v>2694.68292601626</v>
+      </c>
       <c r="E5" s="7"/>
       <c r="F5" s="8" t="s">
         <v>8</v>
       </c>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -1654,11 +1801,15 @@
         <f aca="false">'Snap Leeson'!D15</f>
         <v>5477.19</v>
       </c>
-      <c r="D6" s="6"/>
+      <c r="D6" s="6" t="n">
+        <f aca="false">'Helloprint 24-09'!F13</f>
+        <v>3314.459999</v>
+      </c>
       <c r="E6" s="7"/>
       <c r="F6" s="8"/>
-    </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>10</v>
       </c>
@@ -1671,16 +1822,17 @@
         <v>4129</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">Comparativo!D13</f>
-        <v>1234.37</v>
+        <f aca="false">Comparativo!D14</f>
+        <v>2694.68292601626</v>
       </c>
       <c r="E7" s="11" t="n">
-        <f aca="false">Comparativo!J13</f>
+        <f aca="false">Comparativo!J14</f>
         <v>0</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>11</v>
       </c>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
@@ -1695,14 +1847,15 @@
         <v>949.67</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">Comparativo!D14</f>
-        <v>283.9051</v>
+        <f aca="false">Comparativo!D15</f>
+        <v>619.77707298374</v>
       </c>
       <c r="E8" s="7" t="n">
-        <f aca="false">Comparativo!J14</f>
+        <f aca="false">Comparativo!J15</f>
         <v>0</v>
       </c>
       <c r="F8" s="8"/>
+      <c r="G8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
@@ -1717,16 +1870,17 @@
         <v>5078.67</v>
       </c>
       <c r="D9" s="10" t="n">
-        <f aca="false">Comparativo!D15</f>
-        <v>1518.2751</v>
+        <f aca="false">Comparativo!D16</f>
+        <v>3314.459999</v>
       </c>
       <c r="E9" s="11" t="n">
-        <f aca="false">Comparativo!J15</f>
+        <f aca="false">Comparativo!J16</f>
         <v>0</v>
       </c>
       <c r="F9" s="12"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1743,8 +1897,9 @@
       <c r="F10" s="8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>16</v>
       </c>
@@ -1757,15 +1912,17 @@
         <v>2</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>0</v>
+        <f aca="false">Comparativo!D17</f>
+        <v>2</v>
       </c>
       <c r="E11" s="14" t="n">
-        <f aca="false">Comparativo!J16</f>
+        <f aca="false">Comparativo!J17</f>
         <v>8</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>17</v>
       </c>
+      <c r="G11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
@@ -1774,6 +1931,7 @@
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
@@ -1784,6 +1942,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
@@ -1804,165 +1963,192 @@
       <c r="F14" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="G14" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E15" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>33</v>
+      <c r="D16" s="16" t="s">
+        <v>35</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>39</v>
-      </c>
       <c r="F17" s="8" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>46</v>
+        <v>50</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>50</v>
+        <v>54</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>55</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>57</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>55</v>
+        <v>60</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>61</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>57</v>
+        <v>63</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>59</v>
+        <v>54</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>55</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>67</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>66</v>
+        <v>73</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1972,76 +2158,84 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
+      <c r="A25" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
+      <c r="A26" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
+      <c r="A27" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
+      <c r="A28" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
     </row>
     <row r="29" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
+      <c r="A29" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
     </row>
     <row r="30" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
+      <c r="A30" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
@@ -2050,26 +2244,28 @@
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
+      <c r="A32" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A32:G32"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2099,7 +2295,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2109,7 +2305,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2127,428 +2323,428 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E5" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E5" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E6" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E6" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E7" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E7" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E8" s="18" t="n">
+        <v>103</v>
+      </c>
+      <c r="E8" s="19" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E9" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E9" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E10" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E10" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E11" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E11" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E12" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E12" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E13" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E13" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E14" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="E14" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="E15" s="18" t="n">
+        <v>121</v>
+      </c>
+      <c r="E15" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C16" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>112</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="C17" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>112</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="E17" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="E18" s="18" t="n">
+        <v>121</v>
+      </c>
+      <c r="E18" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="E19" s="18" t="n">
+        <v>129</v>
+      </c>
+      <c r="E19" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="E20" s="18" t="n">
+        <v>129</v>
+      </c>
+      <c r="E20" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="E21" s="18" t="n">
+        <v>129</v>
+      </c>
+      <c r="E21" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="E22" s="18" t="n">
+        <v>134</v>
+      </c>
+      <c r="E22" s="19" t="n">
         <v>16</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="E23" s="18" t="n">
+        <v>139</v>
+      </c>
+      <c r="E23" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E24" s="18" t="n">
+        <v>67</v>
+      </c>
+      <c r="E24" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9"/>
       <c r="B25" s="9" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
@@ -2568,7 +2764,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -2578,22 +2774,22 @@
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2601,21 +2797,21 @@
         <v>1</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C29" s="19" t="n">
+        <v>93</v>
+      </c>
+      <c r="C29" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="D29" s="20" t="n">
+      <c r="D29" s="21" t="n">
         <f aca="false">SUMIF($C$5:$C$24,B29,$E$5:$E$24)</f>
         <v>11</v>
       </c>
-      <c r="E29" s="20" t="n">
+      <c r="E29" s="21" t="n">
         <f aca="false">C29-D29</f>
         <v>1</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2623,9 +2819,9 @@
         <v>2</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="21" t="n">
+        <v>33</v>
+      </c>
+      <c r="C30" s="22" t="n">
         <v>3</v>
       </c>
       <c r="D30" s="5" t="n">
@@ -2643,9 +2839,9 @@
         <v>3</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C31" s="21" t="n">
+        <v>120</v>
+      </c>
+      <c r="C31" s="22" t="n">
         <v>4</v>
       </c>
       <c r="D31" s="5" t="n">
@@ -2657,7 +2853,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2665,9 +2861,9 @@
         <v>4</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C32" s="21" t="n">
+        <v>39</v>
+      </c>
+      <c r="C32" s="22" t="n">
         <v>3</v>
       </c>
       <c r="D32" s="5" t="n">
@@ -2685,9 +2881,9 @@
         <v>5</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C33" s="21" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" s="22" t="n">
         <v>16</v>
       </c>
       <c r="D33" s="5" t="n">
@@ -2705,9 +2901,9 @@
         <v>6</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="C34" s="21" t="n">
+        <v>138</v>
+      </c>
+      <c r="C34" s="22" t="n">
         <v>2</v>
       </c>
       <c r="D34" s="5" t="n">
@@ -2719,7 +2915,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2727,9 +2923,9 @@
         <v>7</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="C35" s="21" t="n">
+        <v>141</v>
+      </c>
+      <c r="C35" s="22" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="5" t="n">
@@ -2741,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9"/>
       <c r="B36" s="9" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="C36" s="9" t="n">
         <f aca="false">SUM(C29:C35)</f>
@@ -2796,7 +2992,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2809,7 +3005,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2833,51 +3029,51 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>141</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>156</v>
-      </c>
-      <c r="B5" s="23" t="n">
+      <c r="A5" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B5" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="25" t="n">
         <v>70</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">B5*C5</f>
         <v>840</v>
       </c>
-      <c r="E5" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="F5" s="25" t="n">
+      <c r="E5" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="F5" s="26" t="n">
         <v>12</v>
       </c>
       <c r="G5" s="6" t="n">
@@ -2889,27 +3085,27 @@
         <v>0</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="B6" s="19" t="n">
+      <c r="A6" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="25" t="n">
         <v>74</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">B6*C6</f>
         <v>888</v>
       </c>
-      <c r="E6" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="20" t="n">
+      <c r="E6" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="21" t="n">
         <v>3</v>
       </c>
       <c r="G6" s="6" t="n">
@@ -2921,27 +3117,27 @@
         <v>-666</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="B7" s="23" t="n">
+      <c r="A7" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="25" t="n">
         <v>149</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">B7*C7</f>
         <v>447</v>
       </c>
-      <c r="E7" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="25" t="n">
+      <c r="E7" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="26" t="n">
         <v>3</v>
       </c>
       <c r="G7" s="6" t="n">
@@ -2953,27 +3149,27 @@
         <v>0</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>162</v>
-      </c>
-      <c r="B8" s="23" t="n">
+      <c r="A8" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="25" t="n">
         <v>99</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">B8*C8</f>
         <v>1584</v>
       </c>
-      <c r="E8" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="25" t="n">
+      <c r="E8" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="26" t="n">
         <v>16</v>
       </c>
       <c r="G8" s="6" t="n">
@@ -2985,28 +3181,28 @@
         <v>0</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="B9" s="19" t="n">
+      <c r="A9" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="B9" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="25" t="n">
         <v>35</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">B9*C9</f>
         <v>140</v>
       </c>
-      <c r="E9" s="26" t="s">
-        <v>165</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>166</v>
+      <c r="E9" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>174</v>
       </c>
       <c r="G9" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F9),F9*C9,"a cotar")</f>
@@ -3017,17 +3213,17 @@
         <v>-140</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="B10" s="21" t="n">
+        <v>176</v>
+      </c>
+      <c r="B10" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="24" t="n">
+      <c r="C10" s="25" t="n">
         <v>15</v>
       </c>
       <c r="D10" s="6" t="n">
@@ -3035,7 +3231,7 @@
         <v>15</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>1</v>
@@ -3049,12 +3245,12 @@
         <v>0</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="B11" s="28" t="n">
         <v>0</v>
@@ -3064,24 +3260,24 @@
         <v>0</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="F11" s="29" t="n">
         <v>2</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B12" s="28" t="n">
         <v>0</v>
@@ -3091,24 +3287,24 @@
         <v>0</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="F12" s="29" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3130,7 +3326,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B14" s="32" t="n">
         <v>0.23</v>
@@ -3154,7 +3350,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -3187,7 +3383,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -3200,7 +3396,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -3213,7 +3409,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3256,7 +3452,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3269,7 +3465,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3293,51 +3489,51 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>141</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>182</v>
-      </c>
-      <c r="B5" s="23" t="n">
+      <c r="A5" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="B5" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="25" t="n">
         <v>110</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">B5*C5</f>
         <v>1320</v>
       </c>
-      <c r="E5" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="F5" s="25" t="n">
+      <c r="E5" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="F5" s="26" t="n">
         <v>12</v>
       </c>
       <c r="G5" s="6" t="n">
@@ -3349,27 +3545,27 @@
         <v>0</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="26" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="19" t="n">
+      <c r="A6" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="25" t="n">
         <v>110</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">B6*C6</f>
         <v>1320</v>
       </c>
-      <c r="E6" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="20" t="n">
+      <c r="E6" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="21" t="n">
         <v>3</v>
       </c>
       <c r="G6" s="6" t="n">
@@ -3381,27 +3577,27 @@
         <v>-990</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="s">
-        <v>186</v>
-      </c>
-      <c r="B7" s="19" t="n">
+      <c r="A7" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="B7" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="25" t="n">
         <v>333</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">B7*C7</f>
         <v>333</v>
       </c>
-      <c r="E7" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="20" t="n">
+      <c r="E7" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="21" t="n">
         <v>3</v>
       </c>
       <c r="G7" s="6" t="n">
@@ -3413,27 +3609,27 @@
         <v>666</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>188</v>
-      </c>
-      <c r="B8" s="23" t="n">
+      <c r="A8" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="B8" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="25" t="n">
         <v>90</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">B8*C8</f>
         <v>1440</v>
       </c>
-      <c r="E8" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="25" t="n">
+      <c r="E8" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="26" t="n">
         <v>16</v>
       </c>
       <c r="G8" s="6" t="n">
@@ -3445,17 +3641,17 @@
         <v>0</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="B9" s="21" t="n">
+        <v>198</v>
+      </c>
+      <c r="B9" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="25" t="n">
         <v>154.6875</v>
       </c>
       <c r="D9" s="6" t="n">
@@ -3463,7 +3659,7 @@
         <v>2475</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>0</v>
@@ -3472,30 +3668,30 @@
         <v>0</v>
       </c>
       <c r="H9" s="31" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
-        <v>194</v>
-      </c>
-      <c r="B10" s="23" t="n">
+      <c r="A10" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="B10" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="24" t="n">
+      <c r="C10" s="25" t="n">
         <v>20</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">B10*C10</f>
         <v>40</v>
       </c>
-      <c r="E10" s="22" t="s">
-        <v>130</v>
-      </c>
-      <c r="F10" s="25" t="n">
+      <c r="E10" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="F10" s="26" t="n">
         <v>2</v>
       </c>
       <c r="G10" s="6" t="n">
@@ -3507,12 +3703,12 @@
         <v>0</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B11" s="28" t="n">
         <v>0</v>
@@ -3522,24 +3718,24 @@
         <v>0</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="F11" s="29" t="n">
         <v>4</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B12" s="28" t="n">
         <v>0</v>
@@ -3549,24 +3745,24 @@
         <v>0</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="F12" s="29" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3588,7 +3784,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B14" s="32" t="n">
         <v>0.23</v>
@@ -3612,7 +3808,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -3645,7 +3841,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -3658,7 +3854,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -3671,7 +3867,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3695,6 +3891,443 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>146.36</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <f aca="false">C5*D5*E5</f>
+        <v>439.08</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <f aca="false">E5/(1+$E$14)</f>
+        <v>118.991869918699</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <f aca="false">C5*D5*G5</f>
+        <v>356.975609756098</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>104.54</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <f aca="false">C6*D6*E6</f>
+        <v>1672.64</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <f aca="false">E6/(1+$E$14)</f>
+        <v>84.9918699186992</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <f aca="false">C6*D6*G6</f>
+        <v>1359.86991869919</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <f aca="false">C7*D7*E7</f>
+        <v>1121.64</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <f aca="false">E7/(1+$E$14)</f>
+        <v>75.9918699186992</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <f aca="false">C7*D7*G7</f>
+        <v>911.90243902439</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>42.913333</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <f aca="false">C8*D8*E8</f>
+        <v>128.739999</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <f aca="false">E8/(1+$E$14)</f>
+        <v>34.8888886178862</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <f aca="false">C8*D8*G8</f>
+        <v>104.666665853659</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>37.68</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <f aca="false">C9*D9*E9</f>
+        <v>75.36</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <f aca="false">E9/(1+$E$14)</f>
+        <v>30.6341463414634</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <f aca="false">C9*D9*G9</f>
+        <v>61.2682926829268</v>
+      </c>
+      <c r="I9" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="10" t="n">
+        <f aca="false">SUM(F5:F9)</f>
+        <v>3437.459999</v>
+      </c>
+      <c r="G10" s="9"/>
+      <c r="H10" s="10" t="n">
+        <f aca="false">SUM(H5:H9)</f>
+        <v>2794.68292601626</v>
+      </c>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="33" t="n">
+        <v>-123</v>
+      </c>
+      <c r="G11" s="9"/>
+      <c r="H11" s="10" t="n">
+        <f aca="false">F11/(1+$E$14)</f>
+        <v>-100</v>
+      </c>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="9"/>
+      <c r="H12" s="10" t="n">
+        <f aca="false">F12/(1+$E$14)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="10" t="n">
+        <f aca="false">F10+F11+F12</f>
+        <v>3314.459999</v>
+      </c>
+      <c r="G13" s="9"/>
+      <c r="H13" s="10" t="n">
+        <f aca="false">H10+H11+H12</f>
+        <v>2694.68292601626</v>
+      </c>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="34" t="s">
+        <v>240</v>
+      </c>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="35" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="F14" s="36" t="n">
+        <f aca="false">F13-H13</f>
+        <v>619.77707298374</v>
+      </c>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="34" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="37" t="s">
+        <v>242</v>
+      </c>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="37"/>
+    </row>
+    <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="37" t="s">
+        <v>243</v>
+      </c>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="37"/>
+    </row>
+    <row r="18" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="37" t="s">
+        <v>244</v>
+      </c>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="37"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A18:J18"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3715,7 +4348,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>245</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3729,7 +4362,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>203</v>
+        <v>246</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3755,56 +4388,56 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>204</v>
+        <v>247</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>205</v>
+        <v>248</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>206</v>
+        <v>249</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>207</v>
+        <v>250</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>208</v>
+        <v>251</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>209</v>
+        <v>252</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>212</v>
+        <v>253</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="D5" s="33" t="s">
-        <v>214</v>
+        <v>254</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>255</v>
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">Necessidade!$C$29</f>
         <v>12</v>
       </c>
-      <c r="F5" s="34"/>
-      <c r="G5" s="35" t="s">
-        <v>215</v>
+      <c r="F5" s="39"/>
+      <c r="G5" s="40" t="s">
+        <v>256</v>
       </c>
       <c r="H5" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F5),IF(UPPER(G5)="S",F5/(1+$B$17),F5),"")</f>
@@ -3815,29 +4448,29 @@
         <v/>
       </c>
       <c r="J5" s="8" t="s">
-        <v>216</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>217</v>
+        <v>258</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="D6" s="33" t="s">
-        <v>219</v>
+        <v>259</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>260</v>
       </c>
       <c r="E6" s="5" t="n">
         <f aca="false">Necessidade!$C$30</f>
         <v>3</v>
       </c>
-      <c r="F6" s="34"/>
-      <c r="G6" s="35" t="s">
-        <v>215</v>
+      <c r="F6" s="39"/>
+      <c r="G6" s="40" t="s">
+        <v>256</v>
       </c>
       <c r="H6" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F6),IF(UPPER(G6)="S",F6/(1+$B$17),F6),"")</f>
@@ -3848,28 +4481,28 @@
         <v/>
       </c>
       <c r="J6" s="8" t="s">
-        <v>220</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>221</v>
+        <v>262</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>222</v>
+        <v>263</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>224</v>
+        <v>264</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>265</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="34"/>
-      <c r="G7" s="35" t="s">
-        <v>215</v>
+      <c r="F7" s="39"/>
+      <c r="G7" s="40" t="s">
+        <v>256</v>
       </c>
       <c r="H7" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F7),IF(UPPER(G7)="S",F7/(1+$B$17),F7),"")</f>
@@ -3880,28 +4513,28 @@
         <v/>
       </c>
       <c r="J7" s="8" t="s">
-        <v>225</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>226</v>
+        <v>267</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>227</v>
+        <v>268</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>228</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>229</v>
+        <v>269</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>270</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="34"/>
-      <c r="G8" s="35" t="s">
-        <v>215</v>
+      <c r="F8" s="39"/>
+      <c r="G8" s="40" t="s">
+        <v>256</v>
       </c>
       <c r="H8" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F8),IF(UPPER(G8)="S",F8/(1+$B$17),F8),"")</f>
@@ -3912,29 +4545,29 @@
         <v/>
       </c>
       <c r="J8" s="8" t="s">
-        <v>230</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>231</v>
+        <v>272</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="D9" s="33" t="s">
-        <v>233</v>
+        <v>273</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>274</v>
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">Necessidade!$C$32</f>
         <v>3</v>
       </c>
-      <c r="F9" s="34"/>
-      <c r="G9" s="35" t="s">
-        <v>215</v>
+      <c r="F9" s="39"/>
+      <c r="G9" s="40" t="s">
+        <v>256</v>
       </c>
       <c r="H9" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F9),IF(UPPER(G9)="S",F9/(1+$B$17),F9),"")</f>
@@ -3945,29 +4578,29 @@
         <v/>
       </c>
       <c r="J9" s="8" t="s">
-        <v>234</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>231</v>
+        <v>272</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="D10" s="33" t="s">
-        <v>233</v>
+        <v>276</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>274</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">Necessidade!$C$33</f>
         <v>16</v>
       </c>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35" t="s">
-        <v>215</v>
+      <c r="F10" s="39"/>
+      <c r="G10" s="40" t="s">
+        <v>256</v>
       </c>
       <c r="H10" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F10),IF(UPPER(G10)="S",F10/(1+$B$17),F10),"")</f>
@@ -3978,29 +4611,29 @@
         <v/>
       </c>
       <c r="J10" s="8" t="s">
-        <v>236</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>237</v>
+        <v>278</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="D11" s="33" t="s">
-        <v>239</v>
+        <v>279</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>280</v>
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">Necessidade!$C$34</f>
         <v>2</v>
       </c>
-      <c r="F11" s="34"/>
-      <c r="G11" s="35" t="s">
-        <v>215</v>
+      <c r="F11" s="39"/>
+      <c r="G11" s="40" t="s">
+        <v>256</v>
       </c>
       <c r="H11" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F11),IF(UPPER(G11)="S",F11/(1+$B$17),F11),"")</f>
@@ -4011,51 +4644,51 @@
         <v/>
       </c>
       <c r="J11" s="8" t="s">
-        <v>240</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>241</v>
+        <v>282</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5" t="n">
         <f aca="false">Necessidade!$C$35</f>
         <v>1</v>
       </c>
-      <c r="F12" s="24"/>
-      <c r="G12" s="36"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="41"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="8" t="s">
-        <v>242</v>
+        <v>283</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="D13" s="33" t="s">
-        <v>245</v>
+        <v>284</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>285</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="34"/>
-      <c r="G13" s="35" t="s">
-        <v>215</v>
+      <c r="F13" s="39"/>
+      <c r="G13" s="40" t="s">
+        <v>256</v>
       </c>
       <c r="H13" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F13),IF(UPPER(G13)="S",F13/(1+$B$17),F13),"")</f>
@@ -4066,12 +4699,12 @@
         <v/>
       </c>
       <c r="J13" s="8" t="s">
-        <v>246</v>
+        <v>286</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>247</v>
+        <v>287</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -4088,7 +4721,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -4105,7 +4738,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -4121,37 +4754,37 @@
       <c r="J16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37" t="s">
-        <v>248</v>
-      </c>
-      <c r="B17" s="38" t="n">
+      <c r="A17" s="34" t="s">
+        <v>288</v>
+      </c>
+      <c r="B17" s="35" t="n">
         <v>0.23</v>
       </c>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="37"/>
-      <c r="I17" s="37"/>
-      <c r="J17" s="37"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="34"/>
+      <c r="J17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37" t="s">
-        <v>249</v>
-      </c>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="37" t="n">
+      <c r="A18" s="34" t="s">
+        <v>289</v>
+      </c>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="34" t="n">
         <f aca="false">COUNTBLANK(F5:F13)-1</f>
         <v>8</v>
       </c>
-      <c r="J18" s="37"/>
+      <c r="J18" s="34"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
@@ -4166,46 +4799,46 @@
       <c r="J19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="39" t="s">
-        <v>250</v>
-      </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="39"/>
-      <c r="I20" s="39"/>
-      <c r="J20" s="39"/>
+      <c r="A20" s="37" t="s">
+        <v>290</v>
+      </c>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="37"/>
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="39" t="s">
-        <v>251</v>
-      </c>
-      <c r="B21" s="39"/>
-      <c r="C21" s="39"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="39"/>
-      <c r="I21" s="39"/>
-      <c r="J21" s="39"/>
+      <c r="A21" s="37" t="s">
+        <v>291</v>
+      </c>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="37"/>
     </row>
     <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="39" t="s">
-        <v>252</v>
-      </c>
-      <c r="B22" s="39"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="39"/>
-      <c r="H22" s="39"/>
-      <c r="I22" s="39"/>
-      <c r="J22" s="39"/>
+      <c r="A22" s="37" t="s">
+        <v>292</v>
+      </c>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="37"/>
+      <c r="J22" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4234,12 +4867,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -4252,7 +4885,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>253</v>
+        <v>293</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4267,7 +4900,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>254</v>
+        <v>294</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4295,69 +4928,70 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>255</v>
+        <v>295</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>256</v>
+        <v>296</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>257</v>
+        <v>297</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>258</v>
+        <v>298</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>259</v>
+        <v>299</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>260</v>
+        <v>300</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>261</v>
+        <v>301</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>262</v>
+        <v>302</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>263</v>
+        <v>303</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">Necessidade!$C$29</f>
         <v>12</v>
       </c>
-      <c r="C5" s="24" t="n">
-        <v>32.4</v>
+      <c r="C5" s="42" t="n">
+        <f aca="false">IF(ISNUMBER('Helloprint 24-09'!$G$7),'Helloprint 24-09'!$G$7,"")</f>
+        <v>75.9918699186992</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C5),$B5*C5,"")</f>
-        <v>388.8</v>
-      </c>
-      <c r="E5" s="24" t="n">
+        <v>911.90243902439</v>
+      </c>
+      <c r="E5" s="25" t="n">
         <v>70</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E5),$B5*E5,"")</f>
         <v>840</v>
       </c>
-      <c r="G5" s="24" t="n">
+      <c r="G5" s="25" t="n">
         <v>110</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G5),$B5*G5,"")</f>
         <v>1320</v>
       </c>
-      <c r="I5" s="40" t="str">
+      <c r="I5" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$5),Vistaprint!$H$5,"")</f>
         <v/>
       </c>
@@ -4366,39 +5000,40 @@
         <v/>
       </c>
       <c r="K5" s="8" t="s">
-        <v>264</v>
+        <v>304</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">Necessidade!$C$30</f>
         <v>3</v>
       </c>
-      <c r="C6" s="24" t="n">
-        <v>55</v>
+      <c r="C6" s="42" t="n">
+        <f aca="false">IF(ISNUMBER('Helloprint 24-09'!$G$8),'Helloprint 24-09'!$G$8,"")</f>
+        <v>34.8888886178862</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C6),$B6*C6,"")</f>
-        <v>165</v>
-      </c>
-      <c r="E6" s="24" t="n">
+        <v>104.666665853659</v>
+      </c>
+      <c r="E6" s="25" t="n">
         <v>74</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E6),$B6*E6,"")</f>
         <v>222</v>
       </c>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="25" t="n">
         <v>110</v>
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G6),$B6*G6,"")</f>
         <v>330</v>
       </c>
-      <c r="I6" s="40" t="str">
+      <c r="I6" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$6),Vistaprint!$H$6,"")</f>
         <v/>
       </c>
@@ -4407,35 +5042,33 @@
         <v/>
       </c>
       <c r="K6" s="8" t="s">
-        <v>265</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">Necessidade!$C$31</f>
         <v>4</v>
       </c>
-      <c r="C7" s="24" t="n">
-        <v>30</v>
-      </c>
-      <c r="D7" s="6" t="n">
+      <c r="C7" s="44"/>
+      <c r="D7" s="45" t="str">
         <f aca="false">IF(ISNUMBER(C7),$B7*C7,"")</f>
-        <v>120</v>
-      </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="42" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="46"/>
+      <c r="F7" s="45" t="str">
         <f aca="false">IF(ISNUMBER(E7),$B7*E7,"")</f>
         <v/>
       </c>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42" t="str">
+      <c r="G7" s="46"/>
+      <c r="H7" s="45" t="str">
         <f aca="false">IF(ISNUMBER(G7),$B7*G7,"")</f>
         <v/>
       </c>
-      <c r="I7" s="40" t="str">
+      <c r="I7" s="43" t="str">
         <f aca="false">IF(AND(ISNUMBER(Vistaprint!$H$7),ISNUMBER(Vistaprint!$H$8)),(Vistaprint!$I$7+Vistaprint!$I$8)/(Vistaprint!$E$7+Vistaprint!$E$8),"")</f>
         <v/>
       </c>
@@ -4444,39 +5077,40 @@
         <v/>
       </c>
       <c r="K7" s="8" t="s">
-        <v>266</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">Necessidade!$C$32</f>
         <v>3</v>
       </c>
-      <c r="C8" s="24" t="n">
-        <v>30.86</v>
+      <c r="C8" s="42" t="n">
+        <f aca="false">IF(ISNUMBER('Helloprint 24-09'!$G$5),'Helloprint 24-09'!$G$5,"")</f>
+        <v>118.991869918699</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C8),$B8*C8,"")</f>
-        <v>92.58</v>
-      </c>
-      <c r="E8" s="24" t="n">
+        <v>356.975609756098</v>
+      </c>
+      <c r="E8" s="25" t="n">
         <v>149</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E8),$B8*E8,"")</f>
         <v>447</v>
       </c>
-      <c r="G8" s="24" t="n">
+      <c r="G8" s="25" t="n">
         <v>333</v>
       </c>
       <c r="H8" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G8),$B8*G8,"")</f>
         <v>999</v>
       </c>
-      <c r="I8" s="40" t="str">
+      <c r="I8" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$9),Vistaprint!$H$9,"")</f>
         <v/>
       </c>
@@ -4485,39 +5119,40 @@
         <v/>
       </c>
       <c r="K8" s="8" t="s">
-        <v>267</v>
+        <v>307</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">Necessidade!$C$33</f>
         <v>16</v>
       </c>
-      <c r="C9" s="24" t="n">
-        <v>24.874375</v>
+      <c r="C9" s="42" t="n">
+        <f aca="false">IF(ISNUMBER('Helloprint 24-09'!$G$6),'Helloprint 24-09'!$G$6,"")</f>
+        <v>84.9918699186992</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C9),$B9*C9,"")</f>
-        <v>397.99</v>
-      </c>
-      <c r="E9" s="24" t="n">
+        <v>1359.86991869919</v>
+      </c>
+      <c r="E9" s="25" t="n">
         <v>99</v>
       </c>
       <c r="F9" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E9),$B9*E9,"")</f>
         <v>1584</v>
       </c>
-      <c r="G9" s="24" t="n">
+      <c r="G9" s="25" t="n">
         <v>90</v>
       </c>
       <c r="H9" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G9),$B9*G9,"")</f>
         <v>1440</v>
       </c>
-      <c r="I9" s="40" t="str">
+      <c r="I9" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$10),Vistaprint!$H$10,"")</f>
         <v/>
       </c>
@@ -4526,37 +5161,38 @@
         <v/>
       </c>
       <c r="K9" s="8" t="s">
-        <v>268</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Necessidade!$C$34</f>
         <v>2</v>
       </c>
-      <c r="C10" s="24" t="n">
-        <v>15</v>
+      <c r="C10" s="42" t="n">
+        <f aca="false">IF(ISNUMBER('Helloprint 24-09'!$G$9),'Helloprint 24-09'!$G$9,"")</f>
+        <v>30.6341463414634</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C10),$B10*C10,"")</f>
-        <v>30</v>
-      </c>
-      <c r="E10" s="41"/>
-      <c r="F10" s="42" t="str">
+        <v>61.2682926829268</v>
+      </c>
+      <c r="E10" s="46"/>
+      <c r="F10" s="45" t="str">
         <f aca="false">IF(ISNUMBER(E10),$B10*E10,"")</f>
         <v/>
       </c>
-      <c r="G10" s="24" t="n">
+      <c r="G10" s="25" t="n">
         <v>20</v>
       </c>
       <c r="H10" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G10),$B10*G10,"")</f>
         <v>40</v>
       </c>
-      <c r="I10" s="40" t="str">
+      <c r="I10" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$11),Vistaprint!$H$11,"")</f>
         <v/>
       </c>
@@ -4565,70 +5201,69 @@
         <v/>
       </c>
       <c r="K10" s="8" t="s">
-        <v>269</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">Necessidade!$C$35</f>
         <v>1</v>
       </c>
-      <c r="C11" s="24" t="n">
-        <v>40</v>
-      </c>
-      <c r="D11" s="6" t="n">
+      <c r="C11" s="44"/>
+      <c r="D11" s="45" t="str">
         <f aca="false">IF(ISNUMBER(C11),$B11*C11,"")</f>
-        <v>40</v>
-      </c>
-      <c r="E11" s="41"/>
-      <c r="F11" s="42" t="str">
+        <v/>
+      </c>
+      <c r="E11" s="46"/>
+      <c r="F11" s="45" t="str">
         <f aca="false">IF(ISNUMBER(E11),$B11*E11,"")</f>
         <v/>
       </c>
-      <c r="G11" s="41"/>
-      <c r="H11" s="42" t="str">
+      <c r="G11" s="46"/>
+      <c r="H11" s="45" t="str">
         <f aca="false">IF(ISNUMBER(G11),$B11*G11,"")</f>
         <v/>
       </c>
-      <c r="I11" s="43"/>
-      <c r="J11" s="42" t="str">
+      <c r="I11" s="44"/>
+      <c r="J11" s="45" t="str">
         <f aca="false">IF(ISNUMBER(I11),$B11*I11,"")</f>
         <v/>
       </c>
       <c r="K11" s="8" t="s">
-        <v>270</v>
+        <v>310</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="24" t="n">
+      <c r="C12" s="42" t="n">
+        <f aca="false">'Helloprint 24-09'!$H$12</f>
         <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">IF(ISNUMBER(C12),$B12*C12,"")</f>
         <v>0</v>
       </c>
-      <c r="E12" s="24" t="n">
+      <c r="E12" s="25" t="n">
         <v>15</v>
       </c>
       <c r="F12" s="6" t="n">
         <f aca="false">IF(ISNUMBER(E12),$B12*E12,"")</f>
         <v>15</v>
       </c>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42" t="str">
+      <c r="G12" s="46"/>
+      <c r="H12" s="45" t="str">
         <f aca="false">IF(ISNUMBER(G12),$B12*G12,"")</f>
         <v/>
       </c>
-      <c r="I12" s="40" t="str">
+      <c r="I12" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$13),Vistaprint!$H$13,"")</f>
         <v/>
       </c>
@@ -4637,160 +5272,185 @@
         <v/>
       </c>
       <c r="K12" s="5" t="s">
-        <v>271</v>
+        <v>311</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10" t="n">
-        <f aca="false">SUM(D5:D12)</f>
-        <v>1234.37</v>
-      </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="10" t="n">
-        <f aca="false">SUM(F5:F12)</f>
-        <v>3108</v>
-      </c>
-      <c r="G13" s="9"/>
-      <c r="H13" s="10" t="n">
-        <f aca="false">SUM(H5:H12)</f>
-        <v>4129</v>
-      </c>
-      <c r="I13" s="9"/>
-      <c r="J13" s="10" t="n">
-        <f aca="false">SUM(J5:J12)</f>
+      <c r="A13" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="42" t="n">
+        <f aca="false">'Helloprint 24-09'!$H$11</f>
+        <v>-100</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(C13),$B13*C13,"")</f>
+        <v>-100</v>
+      </c>
+      <c r="E13" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="9"/>
+      <c r="F13" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E13),$B13*E13,"")</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(G13),$B13*G13,"")</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(I13),$B13*I13,"")</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="B14" s="32" t="n">
-        <v>0.23</v>
-      </c>
+        <v>314</v>
+      </c>
+      <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="10" t="n">
-        <f aca="false">D13*$B$14</f>
-        <v>283.9051</v>
+        <f aca="false">SUM(D5:D13)</f>
+        <v>2694.68292601626</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="10" t="n">
-        <f aca="false">F13*$B$14</f>
-        <v>714.84</v>
+        <f aca="false">SUM(F5:F13)</f>
+        <v>3108</v>
       </c>
       <c r="G14" s="9"/>
       <c r="H14" s="10" t="n">
-        <f aca="false">H13*$B$14</f>
-        <v>949.67</v>
+        <f aca="false">SUM(H5:H13)</f>
+        <v>4129</v>
       </c>
       <c r="I14" s="9"/>
       <c r="J14" s="10" t="n">
-        <f aca="false">J13*$B$14</f>
+        <f aca="false">SUM(J5:J13)</f>
         <v>0</v>
       </c>
       <c r="K14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="B15" s="9"/>
+        <v>183</v>
+      </c>
+      <c r="B15" s="32" t="n">
+        <v>0.23</v>
+      </c>
       <c r="C15" s="9"/>
       <c r="D15" s="10" t="n">
-        <f aca="false">D13+D14</f>
-        <v>1518.2751</v>
+        <f aca="false">D14*$B$15</f>
+        <v>619.77707298374</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="10" t="n">
-        <f aca="false">F13+F14</f>
-        <v>3822.84</v>
+        <f aca="false">F14*$B$15</f>
+        <v>714.84</v>
       </c>
       <c r="G15" s="9"/>
       <c r="H15" s="10" t="n">
-        <f aca="false">H13+H14</f>
-        <v>5078.67</v>
+        <f aca="false">H14*$B$15</f>
+        <v>949.67</v>
       </c>
       <c r="I15" s="9"/>
       <c r="J15" s="10" t="n">
-        <f aca="false">J13+J14</f>
+        <f aca="false">J14*$B$15</f>
         <v>0</v>
       </c>
       <c r="K15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="37" t="s">
-        <v>273</v>
-      </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="37" t="n">
-        <f aca="false">COUNTBLANK(C5:C12)</f>
+      <c r="A16" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="10" t="n">
+        <f aca="false">D14+D15</f>
+        <v>3314.459999</v>
+      </c>
+      <c r="E16" s="9"/>
+      <c r="F16" s="10" t="n">
+        <f aca="false">F14+F15</f>
+        <v>3822.84</v>
+      </c>
+      <c r="G16" s="9"/>
+      <c r="H16" s="10" t="n">
+        <f aca="false">H14+H15</f>
+        <v>5078.67</v>
+      </c>
+      <c r="I16" s="9"/>
+      <c r="J16" s="10" t="n">
+        <f aca="false">J14+J15</f>
         <v>0</v>
       </c>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37" t="n">
-        <f aca="false">COUNTBLANK(E5:E12)</f>
+      <c r="K16" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="34" t="s">
+        <v>315</v>
+      </c>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34" t="n">
+        <f aca="false">COUNTBLANK(C5:C13)</f>
+        <v>2</v>
+      </c>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34" t="n">
+        <f aca="false">COUNTBLANK(E5:E13)</f>
         <v>3</v>
       </c>
-      <c r="G16" s="37"/>
-      <c r="H16" s="37" t="n">
-        <f aca="false">COUNTBLANK(G5:G12)</f>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34" t="n">
+        <f aca="false">COUNTBLANK(G5:G13)</f>
         <v>3</v>
       </c>
-      <c r="I16" s="37"/>
-      <c r="J16" s="37" t="n">
-        <f aca="false">COUNTBLANK(I5:I12)</f>
+      <c r="I17" s="34"/>
+      <c r="J17" s="34" t="n">
+        <f aca="false">COUNTBLANK(I5:I13)</f>
         <v>8</v>
       </c>
-      <c r="K16" s="37"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37" t="s">
-        <v>274</v>
-      </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="44" t="n">
-        <f aca="false">IFERROR(F13/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(E5:E12)),"")</f>
-        <v>2.97595679692063</v>
-      </c>
-      <c r="G17" s="37"/>
-      <c r="H17" s="44" t="n">
-        <f aca="false">IFERROR(H13/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(G5:G12)),"")</f>
-        <v>3.84318251626535</v>
-      </c>
-      <c r="I17" s="37"/>
-      <c r="J17" s="44" t="str">
-        <f aca="false">IFERROR(J13/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(I5:I12)),"")</f>
+      <c r="K17" s="34"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="34" t="s">
+        <v>316</v>
+      </c>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="47" t="n">
+        <f aca="false">IFERROR(SUMPRODUCT(($B$5:$B$12)*(E5:E12)*ISNUMBER($C$5:$C$12))/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(E5:E12)),"")</f>
+        <v>1.13703935074419</v>
+      </c>
+      <c r="G18" s="34"/>
+      <c r="H18" s="47" t="n">
+        <f aca="false">IFERROR(SUMPRODUCT(($B$5:$B$12)*(G5:G12)*ISNUMBER($C$5:$C$12))/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(G5:G12)),"")</f>
+        <v>1.47744846528467</v>
+      </c>
+      <c r="I18" s="34"/>
+      <c r="J18" s="47" t="str">
+        <f aca="false">IFERROR(SUMPRODUCT(($B$5:$B$12)*(I5:I12)*ISNUMBER($C$5:$C$12))/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(I5:I12)),"")</f>
         <v/>
       </c>
-      <c r="K17" s="37"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
+      <c r="K18" s="34"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>275</v>
-      </c>
+      <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -4804,7 +5464,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>276</v>
+        <v>317</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -4819,7 +5479,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>277</v>
+        <v>318</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -4834,7 +5494,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>278</v>
+        <v>319</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -4847,6 +5507,21 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Orçamentos: revisão da proposta Snap 1554129 (opção Basic) no comparativo
A aba Snap Leeson passa a ler a proposta revisada de 24/09: 11 fence banners
(€ 1.235), 4 pull-ups largos (€ 1.120), 16 Basic (€ 1.440), 2 corriboard A2
(€ 40), 4 adesivos laminados 900 × 900 (€ 280) e entrega (€ 30) — € 4.145,00
sem IVA, € 5.098,35 com IVA; Premium seria € 5.180,00 / € 6.371,40. A revisão
perdeu os 3 banners PVC 2000 × 1000 da lateral leste e trouxe um 4º pull-up
largo que o plano não tem; os dois pontos ficam marcados na planilha.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1FDufm2zVw9d1c3PLPuzV
</commit_message>
<xml_diff>
--- a/Orçamentos/Sinalização/comparativo_cotacoes_2026-09-24.xlsx
+++ b/Orçamentos/Sinalização/comparativo_cotacoes_2026-09-24.xlsx
@@ -53,7 +53,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="D13" authorId="0">
+    <comment ref="D14" authorId="0">
       <text>
         <r>
           <rPr>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="326">
   <si>
     <t xml:space="preserve">Cotações de sinalização × necessidade do plano — 24/09/2026</t>
   </si>
@@ -103,7 +103,7 @@
     <t xml:space="preserve">Banner Printing (e-mail)</t>
   </si>
   <si>
-    <t xml:space="preserve">Snap Leeson (ref. 1554129)</t>
+    <t xml:space="preserve">Snap Leeson (1554129 revisada, Basic)</t>
   </si>
   <si>
     <t xml:space="preserve">Helloprint (carrinho 24/09)</t>
@@ -145,7 +145,7 @@
     <t xml:space="preserve">Linhas ainda por cotar</t>
   </si>
   <si>
-    <t xml:space="preserve">Banner Printing: vinil, correx, fixação. Snap: vinil, fixação. Helloprint: vinil, fixação. Vistaprint: as linhas cujo preço ainda não foi colado.</t>
+    <t xml:space="preserve">Banner Printing: vinil, correx, fixação. Snap: PVC 2000 × 1000 (saiu da revisão), fixação. Helloprint: vinil, fixação. Vistaprint: as linhas cujo preço ainda não foi colado.</t>
   </si>
   <si>
     <t xml:space="preserve">O que dizer a cada gráfica</t>
@@ -157,7 +157,7 @@
     <t xml:space="preserve">Banner Printing</t>
   </si>
   <si>
-    <t xml:space="preserve">Snap Leeson</t>
+    <t xml:space="preserve">Snap Leeson (revisada)</t>
   </si>
   <si>
     <t xml:space="preserve">Helloprint carrinho 24/09</t>
@@ -178,7 +178,7 @@
     <t xml:space="preserve">12 × € 70</t>
   </si>
   <si>
-    <t xml:space="preserve">12 × € 110 (lote € 1.320)</t>
+    <t xml:space="preserve">11 (lote € 1.235 = € 112,27/un)</t>
   </si>
   <si>
     <t xml:space="preserve">12 × € 93,47 c/ IVA (RPET 208 × 82, linhas de 1)</t>
@@ -190,7 +190,7 @@
     <t xml:space="preserve">mesh 208 × 82 cm personalizado</t>
   </si>
   <si>
-    <t xml:space="preserve">Nada a corrigir no pedido. Internamente: confirmar 12 × 11 antes de fechar. Helloprint: RPET, não mesh — conferir se serve no gradil.</t>
+    <t xml:space="preserve">Snap já está em 11, que é o que as fichas do artefato somam. Decidir 11 ou 12 e alinhar Banner Printing e Helloprint ao mesmo número. Helloprint: RPET, não mesh — conferir se serve no gradil.</t>
   </si>
   <si>
     <t xml:space="preserve">Banner PVC 2000 × 1000 mm</t>
@@ -199,6 +199,9 @@
     <t xml:space="preserve">12 × € 74</t>
   </si>
   <si>
+    <t xml:space="preserve">saiu da revisão (v1: 12 × € 110)</t>
+  </si>
+  <si>
     <t xml:space="preserve">3 × mesh 200 × 82 (linha de € 128,74 c/ IVA) — premissa: é a P2?</t>
   </si>
   <si>
@@ -208,7 +211,7 @@
     <t xml:space="preserve">vinyl banner 100 × 200 cm</t>
   </si>
   <si>
-    <t xml:space="preserve">Reduzir de 12 para 3. As 12 foram copiadas do número de fence banners. Helloprint: se os 3 mesh forem a P2, a arte (2:1) precisa ser refeita para 200 × 82.</t>
+    <t xml:space="preserve">Banner Printing: reduzir de 12 para 3. Snap: pedir a linha de volta, com 3. Helloprint: se os 3 mesh forem a P2, a arte (2:1) precisa ser refeita para 200 × 82.</t>
   </si>
   <si>
     <t xml:space="preserve">Pull-up 1000 × 2000 mm</t>
@@ -217,7 +220,7 @@
     <t xml:space="preserve">3 × € 149</t>
   </si>
   <si>
-    <t xml:space="preserve">1 × € 333</t>
+    <t xml:space="preserve">4 (lote € 1.120 = € 280/un)</t>
   </si>
   <si>
     <t xml:space="preserve">3 × € 146,36 c/ IVA (Medium)</t>
@@ -226,7 +229,7 @@
     <t xml:space="preserve">roller banner 100 × 200 cm</t>
   </si>
   <si>
-    <t xml:space="preserve">Snap: subir de 1 para 3. Banner Printing e Helloprint estão certos.</t>
+    <t xml:space="preserve">Snap: veio 4; o plano prevê 3 — confirmar se o 4º foi pedido de propósito. Banner Printing e Helloprint estão certos.</t>
   </si>
   <si>
     <t xml:space="preserve">Pull-up 850 × 2000 mm</t>
@@ -235,7 +238,7 @@
     <t xml:space="preserve">16 × € 99</t>
   </si>
   <si>
-    <t xml:space="preserve">16 × € 90 (Basic) ou € 154,69 (Premium)</t>
+    <t xml:space="preserve">16 × € 90 (Basic, escolhida) ou € 154,69 (Premium)</t>
   </si>
   <si>
     <t xml:space="preserve">16 × € 104,54 c/ IVA (Small)</t>
@@ -247,7 +250,7 @@
     <t xml:space="preserve">roller banner 85 × 200 cm</t>
   </si>
   <si>
-    <t xml:space="preserve">Nada a corrigir. Snap: escolher Basic ou Premium.</t>
+    <t xml:space="preserve">Nada a corrigir.</t>
   </si>
   <si>
     <t xml:space="preserve">Vinil recortado para vidro 1200 × 700 mm</t>
@@ -256,24 +259,27 @@
     <t xml:space="preserve">4 × "90 × 90 cm custom banner" a € 35</t>
   </si>
   <si>
+    <t xml:space="preserve">4 × adesivo laminado 900 × 900 (lote € 280 = € 70/un)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">não está no carrinho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 × window lettering (≤ 50 × 50 cm) + 1 × window decal (S7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banner Printing: trocar o banner 90 × 90 por vinil adesivo recortado (letras A/B/C de 300 mm + pictogramas da S7), removível. Snap: é adesivo impresso 900 × 900, não recortado — aceitar se o fundo opaco servir; conferir remoção sem resíduo. Helloprint: acrescentar ao carrinho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placa correx 4 mm A2 (594 × 420)</t>
+  </si>
+  <si>
     <t xml:space="preserve">não cotado</t>
   </si>
   <si>
-    <t xml:space="preserve">não está no carrinho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 × window lettering (≤ 50 × 50 cm) + 1 × window decal (S7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Banner Printing: trocar o banner 90 × 90 por vinil adesivo recortado (letras A/B/C de 300 mm + pictogramas da S7), removível. Snap: pedir a linha. Helloprint: acrescentar ao carrinho.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placa correx 4 mm A2 (594 × 420)</t>
-  </si>
-  <si>
     <t xml:space="preserve">2 × € 20 (corriboard 5 mm)</t>
   </si>
   <si>
@@ -307,7 +313,7 @@
     <t xml:space="preserve">€ 15</t>
   </si>
   <si>
-    <t xml:space="preserve">não informado</t>
+    <t xml:space="preserve">€ 30 (Donnybrook Road)</t>
   </si>
   <si>
     <t xml:space="preserve">grátis, Standard até 30/09; desconto de € 123 c/ IVA no carrinho</t>
@@ -316,7 +322,7 @@
     <t xml:space="preserve">no checkout (economy / standard / fast)</t>
   </si>
   <si>
-    <t xml:space="preserve">Snap: perguntar frete ou retirada. Prazo: eleição em 04/10. Helloprint: pedir até 21h de 24/09 para manter as datas.</t>
+    <t xml:space="preserve">Prazo: eleição em 04/10. Snap não informou data de entrega. Helloprint: pedir até 21h de 24/09 para manter as datas.</t>
   </si>
   <si>
     <t xml:space="preserve">Ressalvas</t>
@@ -325,10 +331,10 @@
     <t xml:space="preserve">1. Fence banners: a tabela do artefato diz 12 (10 da cotação de 18/09 + 2º P0-Consulta + Fim da avenida B) e "19 peças externas", mas as fichas peça a peça somam 11 (P0 2+2, P1, P3, P4 ×4, P5-Preferencial). Esta planilha usa 12; se for 11, tire um unitário de cada coluna.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Unitários de lote (Snap) reaplicados a quantidades menores são premissa: 3 PVC e 3 pull-ups largos podem sair mais caros por unidade do que 12 e 1. Pedir a cotação refeita, não só multiplicar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Os dois totais corrigidos não incluem o vinil recortado nem a fixação; o da Banner Printing também não inclui as placas correx. Comparar só depois de as gráficas cotarem o que falta.</t>
+    <t xml:space="preserve">2. Snap, revisão de 24/09 (opção Basic): € 4.145,00 sem IVA, € 5.098,35 com IVA; Premium: € 5.180,00 / € 6.371,40. A revisão corrigiu o fence banner para 11 e o pull-up largo para 4, mas perdeu os 3 banners PVC 2000 × 1000 da lateral leste e cotou o vinil das portas como adesivo impresso 900 × 900. O 4º pull-up largo (€ 280) precisa de confirmação: o plano tem 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Os totais corrigidos não incluem o que cada gráfica não cotou: Banner Printing sem vinil, correx e fixação; Snap sem os 3 PVC e a fixação; Helloprint sem vinil e fixação. Comparar só depois de fechar as linhas que faltam.</t>
   </si>
   <si>
     <t xml:space="preserve">4. O carrinho Helloprint de 24/09 (€ 2.694,68 sem IVA, € 3.314,46 com IVA, já com € 100 de desconto) superou a referência de 18/09 (€ 1.234,37): aquela supunha preço de tiragem para peças de arte diferente. Ainda assim fica abaixo da Banner Printing e da Snap nas linhas comparáveis (aba Comparativo, linha "Múltiplo"). Falta nele o vinil das quatro portas, e duas linhas são premissa de leitura: os 3 mesh 200 × 82 como P2 e os 2 stickers 42 × 60 como saídas.</t>
@@ -661,31 +667,25 @@
     <t xml:space="preserve">Snap Leeson — o que foi cotado × o que o plano precisa</t>
   </si>
   <si>
-    <t xml:space="preserve">Proposta ref. 1554129 (Snap Leeson / JK Printing), 24/09/2026 — preços ex VAT</t>
+    <t xml:space="preserve">Proposta ref. 1554129 revisada (Snap Leeson / JK Printing), 24/09/2026 — preços ex VAT, opção Basic</t>
   </si>
   <si>
     <t xml:space="preserve">Fence Banners, mesh, 2080 × 820 mm, hemmed &amp; eyeletted</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantidade certa (pela tabela do artefato; as fichas somam 11 — confirmar). Cotado como lote: 12 por € 1.320,00.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PVC Banners 2000 × 1000 mm, hemmed &amp; eyeletted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERRO: o plano precisa de 3, não 12. Cotado como lote (12 por € 1.320,00); o unitário de € 110 para 3 é premissa — pedir novo preço.</t>
+    <t xml:space="preserve">Revisão: 11 (era 12 a € 110). Lote: 11 por € 1.235,00 = € 112,27/un. Bate com a soma das fichas do artefato (11); a tabela do artefato diz 12 — a coluna "Qtd correta" segue a revisão.</t>
   </si>
   <si>
     <t xml:space="preserve">Wide Pull Up Banner 1000 × 2000 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">ERRO: o plano precisa de 3 (painéis das portas A, B e C); a cotação traz 1. Unitário de € 333 para 3 é premissa.</t>
+    <t xml:space="preserve">Revisão: 4 (era 1 a € 333). O plano prevê 3 painéis de porta (A, B, C). Se o 4º foi pedido de propósito, mudar a qtd correta para 4; senão, avisar a Snap. Lote: 4 por € 1.120,00.</t>
   </si>
   <si>
     <t xml:space="preserve">Basic Pull Up Banners (850 × 2000, non-replaceable stands)</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantidade certa. Lote: 16 por € 1.440,00. Alternativa "Premium" abaixo é OU, não E.</t>
+    <t xml:space="preserve">Quantidade certa. Lote: 16 por € 1.440,00. Opção escolhida.</t>
   </si>
   <si>
     <t xml:space="preserve">Premium Pull Up Banners (alternativa aos Basic)</t>
@@ -706,19 +706,34 @@
     <t xml:space="preserve">Quantidade certa (saídas S2 e S8). 5 mm em vez de 4 mm: serve.</t>
   </si>
   <si>
-    <t xml:space="preserve">(não cotado) 4 × vinil recortado para vidro, 1200 × 700 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Letras A, B, C de 300 mm e pictogramas da S7; removível sem resíduo. Faltou no pedido.</t>
+    <t xml:space="preserve">Laminated Vinyl Labels, 900 × 900 mm, matt laminated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrou como adesivo impresso e laminado de 900 × 900 mm, não vinil recortado de 1200 × 700. Serve no vidro se o Posto aceitar fundo opaco em vez de só a letra; conferir remoção sem resíduo. Lote: 4 por € 280,00.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery (2nd Floor, 36-42 Donnybrook Road, D04 E6X0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frete para o endereço informado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(saiu da cotação) Banner PVC 2000 × 1000 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A v1 tinha 12; a revisão não tem nenhum. O plano precisa de 3 para a lateral leste do Hall 2 (P2). Pedir a linha de volta com 3.</t>
   </si>
   <si>
     <t xml:space="preserve">Verba de ~€ 40 no plano; compra à parte.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fonte: proposta ref. 1554129 de Snap Leeson (JK Printing Ltd T/A Snap, 12 Sir John Rogerson's Quay, Dublin 2), Declan O'Leary, 24/09/2026. Preços ex VAT; sem linha de entrega.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unitários calculados a partir dos totais de lote (€ 1.320 / 12; € 1.440 / 16; € 2.475 / 16; € 40 / 2). Recalcular com lotes menores é premissa: gráficas cobram mais por unidade em tiragem menor.</t>
+    <t xml:space="preserve">Fonte: proposta ref. 1554129 REVISADA de Snap Leeson (JK Printing Ltd T/A Snap), Declan O'Leary, 24/09/2026. Preços ex VAT. A v1 do mesmo dia tinha 12 fence, 12 PVC, 1 wide pull-up e nenhum vinil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção Basic: 1.235 + 1.120 + 1.440 + 40 + 280 + 30 = € 4.145,00 sem IVA; € 5.098,35 com IVA. Opção Premium: + € 1.035,00 = € 5.180,00 sem IVA; € 6.371,40 com IVA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unitários calculados a partir dos totais de lote (€ 1.235 / 11; € 1.120 / 4; € 1.440 / 16; € 2.475 / 16; € 40 / 2; € 280 / 4).</t>
   </si>
   <si>
     <t xml:space="preserve">A proposta diz "print-ready PDF with crop marks and bleed": arte final é por nossa conta.</t>
@@ -1006,16 +1021,16 @@
     <t xml:space="preserve">Vistaprint total</t>
   </si>
   <si>
-    <t xml:space="preserve">Helloprint: RPET 208 × 82, 12 linhas de 1 (€ 93,47 c/ IVA). Snap: € 1.320 / 12. Vistaprint: mesh 208 × 82 cm personalizado. Ref. 18/09: € 32,40.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helloprint: PREMISSA — os 3 mesh 200 × 82 do carrinho lidos como a P2 (formato diferente). Snap: € 1.320 / 12, premissa para 3 un. Ref. 18/09: € 55.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Não está no carrinho nem foi cotado pelas duas gráficas. Vistaprint: 3 window lettering + 1 window decal, média das 4 peças. Ref. 18/09: € 30 (premissa).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helloprint: Medium, 3 linhas de 1 (€ 146,36 c/ IVA). Snap: cotou 1 un.; premissa para 3. Ref. 18/09: € 30,86.</t>
+    <t xml:space="preserve">Helloprint: RPET 208 × 82, 12 linhas de 1 (€ 93,47 c/ IVA). Snap (revisão): € 1.235 / 11 = € 112,27. Vistaprint: mesh 208 × 82 cm personalizado. Ref. 18/09: € 32,40.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: PREMISSA — os 3 mesh 200 × 82 do carrinho lidos como a P2 (formato diferente). Snap: saiu da revisão (v1: € 110). Ref. 18/09: € 55.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snap (revisão): 4 adesivos laminados 900 × 900 a € 280 — impresso, não recortado. Helloprint: não está no carrinho. Banner Printing: cotou banner 90 × 90. Vistaprint: 3 window lettering + 1 window decal, média das 4 peças. Ref. 18/09: € 30 (premissa).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helloprint: Medium, 3 linhas de 1 (€ 146,36 c/ IVA). Snap (revisão): 4 por € 1.120 = € 280/un; o plano prevê 3. Ref. 18/09: € 30,86.</t>
   </si>
   <si>
     <t xml:space="preserve">Helloprint: Small, 16 linhas de 1 (€ 104,54 c/ IVA). Snap "Basic"; a "Premium" sai a € 154,69/un. Ref. 18/09: € 24,87.</t>
@@ -1027,7 +1042,7 @@
     <t xml:space="preserve">Verba de ~€ 40; compra à parte, ninguém cota.</t>
   </si>
   <si>
-    <t xml:space="preserve">Helloprint: grátis (Standard até 30/09). Banner Printing: € 15. Snap: não informou. Vistaprint: frete do checkout, aba Vistaprint.</t>
+    <t xml:space="preserve">Helloprint: grátis (Standard até 30/09). Banner Printing: € 15. Snap (revisão): € 30 para Donnybrook Road. Vistaprint: frete do checkout, aba Vistaprint.</t>
   </si>
   <si>
     <t xml:space="preserve">Desconto do carrinho</t>
@@ -1441,7 +1456,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1449,7 +1464,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1748,7 +1763,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
         <v>2</v>
@@ -1776,8 +1791,8 @@
         <v>3914</v>
       </c>
       <c r="C5" s="6" t="n">
-        <f aca="false">'Snap Leeson'!D13</f>
-        <v>4453</v>
+        <f aca="false">'Snap Leeson'!D14</f>
+        <v>4145</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">'Helloprint 24-09'!H13</f>
@@ -1798,8 +1813,8 @@
         <v>4814.22</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">'Snap Leeson'!D15</f>
-        <v>5477.19</v>
+        <f aca="false">'Snap Leeson'!D16</f>
+        <v>5098.35</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">'Helloprint 24-09'!F13</f>
@@ -1818,8 +1833,8 @@
         <v>3108</v>
       </c>
       <c r="C7" s="10" t="n">
-        <f aca="false">'Snap Leeson'!G13</f>
-        <v>4129</v>
+        <f aca="false">'Snap Leeson'!G14</f>
+        <v>3865</v>
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">Comparativo!D14</f>
@@ -1843,8 +1858,8 @@
         <v>714.84</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">'Snap Leeson'!G14</f>
-        <v>949.67</v>
+        <f aca="false">'Snap Leeson'!G15</f>
+        <v>888.95</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">Comparativo!D15</f>
@@ -1866,8 +1881,8 @@
         <v>3822.84</v>
       </c>
       <c r="C9" s="10" t="n">
-        <f aca="false">'Snap Leeson'!G15</f>
-        <v>5078.67</v>
+        <f aca="false">'Snap Leeson'!G16</f>
+        <v>4753.95</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">Comparativo!D16</f>
@@ -1889,8 +1904,8 @@
         <v>-806</v>
       </c>
       <c r="C10" s="6" t="n">
-        <f aca="false">'Snap Leeson'!H13</f>
-        <v>-324</v>
+        <f aca="false">'Snap Leeson'!H14</f>
+        <v>-280</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="7"/>
@@ -1899,7 +1914,7 @@
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>16</v>
       </c>
@@ -1908,7 +1923,7 @@
         <v>3</v>
       </c>
       <c r="C11" s="13" t="n">
-        <f aca="false">COUNTIF('Snap Leeson'!G5:G12,"a cotar")</f>
+        <f aca="false">COUNTIF('Snap Leeson'!G5:G13,"a cotar")</f>
         <v>2</v>
       </c>
       <c r="D11" s="13" t="n">
@@ -1967,7 +1982,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
         <v>26</v>
       </c>
@@ -1998,157 +2013,157 @@
         <v>34</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F16" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="G16" s="8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>36</v>
-      </c>
       <c r="F17" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>67</v>
-      </c>
       <c r="F22" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2162,7 +2177,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -2173,7 +2188,7 @@
     </row>
     <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -2184,7 +2199,7 @@
     </row>
     <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
@@ -2195,7 +2210,7 @@
     </row>
     <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -2206,7 +2221,7 @@
     </row>
     <row r="28" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -2217,7 +2232,7 @@
     </row>
     <row r="29" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
@@ -2228,7 +2243,7 @@
     </row>
     <row r="30" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
@@ -2248,7 +2263,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="18"/>
       <c r="C32" s="18"/>
@@ -2295,7 +2310,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2305,7 +2320,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2323,428 +2338,428 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E5" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>96</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>94</v>
       </c>
       <c r="E6" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E7" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>33</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E8" s="19" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E9" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E10" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E11" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E12" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E13" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E14" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E15" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B16" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>121</v>
       </c>
       <c r="E16" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E17" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E18" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E19" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B20" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>131</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>129</v>
       </c>
       <c r="E20" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E21" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E22" s="19" t="n">
         <v>16</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E23" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>65</v>
-      </c>
       <c r="C24" s="8" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E24" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9"/>
       <c r="B25" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
@@ -2764,7 +2779,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -2774,22 +2789,22 @@
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2797,7 +2812,7 @@
         <v>1</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C29" s="20" t="n">
         <v>12</v>
@@ -2811,7 +2826,7 @@
         <v>1</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2839,7 +2854,7 @@
         <v>3</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C31" s="22" t="n">
         <v>4</v>
@@ -2853,7 +2868,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2861,7 +2876,7 @@
         <v>4</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C32" s="22" t="n">
         <v>3</v>
@@ -2881,7 +2896,7 @@
         <v>5</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C33" s="22" t="n">
         <v>16</v>
@@ -2901,7 +2916,7 @@
         <v>6</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C34" s="22" t="n">
         <v>2</v>
@@ -2915,7 +2930,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2923,7 +2938,7 @@
         <v>7</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C35" s="22" t="n">
         <v>1</v>
@@ -2937,13 +2952,13 @@
         <v>0</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9"/>
       <c r="B36" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C36" s="9" t="n">
         <f aca="false">SUM(C29:C35)</f>
@@ -2992,7 +3007,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3005,7 +3020,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3029,36 +3044,36 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>12</v>
@@ -3071,7 +3086,7 @@
         <v>840</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F5" s="26" t="n">
         <v>12</v>
@@ -3085,12 +3100,12 @@
         <v>0</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>12</v>
@@ -3117,12 +3132,12 @@
         <v>-666</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B7" s="24" t="n">
         <v>3</v>
@@ -3135,7 +3150,7 @@
         <v>447</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F7" s="26" t="n">
         <v>3</v>
@@ -3149,12 +3164,12 @@
         <v>0</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B8" s="24" t="n">
         <v>16</v>
@@ -3167,7 +3182,7 @@
         <v>1584</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F8" s="26" t="n">
         <v>16</v>
@@ -3181,12 +3196,12 @@
         <v>0</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>4</v>
@@ -3199,10 +3214,10 @@
         <v>140</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G9" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F9),F9*C9,"a cotar")</f>
@@ -3213,12 +3228,12 @@
         <v>-140</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B10" s="22" t="n">
         <v>1</v>
@@ -3231,7 +3246,7 @@
         <v>15</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>1</v>
@@ -3245,12 +3260,12 @@
         <v>0</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B11" s="28" t="n">
         <v>0</v>
@@ -3260,24 +3275,24 @@
         <v>0</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F11" s="29" t="n">
         <v>2</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B12" s="28" t="n">
         <v>0</v>
@@ -3287,24 +3302,24 @@
         <v>0</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F12" s="29" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3326,7 +3341,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B14" s="32" t="n">
         <v>0.23</v>
@@ -3350,7 +3365,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -3383,7 +3398,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -3396,7 +3411,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -3409,7 +3424,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3436,7 +3451,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
@@ -3452,7 +3467,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3465,7 +3480,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3489,253 +3504,258 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B5" s="24" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>110</v>
+        <v>112.272727272727</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">B5*C5</f>
-        <v>1320</v>
+        <v>1235</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(F5),F5*C5,"a cotar")</f>
-        <v>1320</v>
+        <v>1235</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G5),G5-D5,-D5)</f>
         <v>0</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B6" s="20" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">B6*C6</f>
-        <v>1320</v>
+        <v>1120</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="F6" s="21" t="n">
         <v>3</v>
       </c>
       <c r="G6" s="6" t="n">
         <f aca="false">IF(ISNUMBER(F6),F6*C6,"a cotar")</f>
-        <v>330</v>
+        <v>840</v>
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G6),G6-D6,-D6)</f>
-        <v>-990</v>
+        <v>-280</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="B7" s="20" t="n">
-        <v>1</v>
+      <c r="A7" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>16</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>333</v>
+        <v>90</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">B7*C7</f>
-        <v>333</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="21" t="n">
-        <v>3</v>
+        <v>1440</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="26" t="n">
+        <v>16</v>
       </c>
       <c r="G7" s="6" t="n">
         <f aca="false">IF(ISNUMBER(F7),F7*C7,"a cotar")</f>
-        <v>999</v>
+        <v>1440</v>
       </c>
       <c r="H7" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G7),G7-D7,-D7)</f>
-        <v>666</v>
+        <v>0</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="B8" s="24" t="n">
+      <c r="A8" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="B8" s="22" t="n">
         <v>16</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>90</v>
+        <v>154.6875</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">B8*C8</f>
-        <v>1440</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="F8" s="26" t="n">
-        <v>16</v>
+        <v>2475</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G8" s="6" t="n">
-        <f aca="false">IF(ISNUMBER(F8),F8*C8,"a cotar")</f>
-        <v>1440</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <f aca="false">IF(ISNUMBER(G8),G8-D8,-D8)</f>
         <v>0</v>
       </c>
+      <c r="H8" s="31" t="s">
+        <v>200</v>
+      </c>
       <c r="I8" s="8" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="B9" s="22" t="n">
-        <v>16</v>
+        <v>201</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>2</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>154.6875</v>
+        <v>20</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">B9*C9</f>
-        <v>2475</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="F9" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="F9" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(F9),F9*C9,"a cotar")</f>
+        <v>40</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(G9),G9-D9,-D9)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="31" t="s">
-        <v>200</v>
-      </c>
       <c r="I9" s="8" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
-        <v>202</v>
-      </c>
-      <c r="B10" s="24" t="n">
-        <v>2</v>
+        <v>203</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>4</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">B10*C10</f>
-        <v>40</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="F10" s="26" t="n">
-        <v>2</v>
+        <v>280</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>4</v>
       </c>
       <c r="G10" s="6" t="n">
         <f aca="false">IF(ISNUMBER(F10),F10*C10,"a cotar")</f>
-        <v>40</v>
+        <v>280</v>
       </c>
       <c r="H10" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G10),G10-D10,-D10)</f>
         <v>0</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="s">
-        <v>204</v>
-      </c>
-      <c r="B11" s="28" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B11" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <f aca="false">B11*C11</f>
+        <v>30</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(F11),F11*C11,"a cotar")</f>
+        <v>30</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(G11),G11-D11,-D11)</f>
         <v>0</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="29" t="s">
-        <v>173</v>
-      </c>
-      <c r="F11" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="G11" s="30" t="s">
-        <v>174</v>
-      </c>
-      <c r="H11" s="31" t="s">
-        <v>174</v>
-      </c>
       <c r="I11" s="8" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>180</v>
+        <v>208</v>
       </c>
       <c r="B12" s="28" t="n">
         <v>0</v>
@@ -3745,104 +3765,118 @@
         <v>0</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>141</v>
+        <v>33</v>
       </c>
       <c r="F12" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="30" t="s">
+        <v>176</v>
+      </c>
+      <c r="H12" s="31" t="s">
+        <v>176</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="27" t="s">
+        <v>182</v>
+      </c>
+      <c r="B13" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="F13" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="30" t="s">
-        <v>174</v>
-      </c>
-      <c r="H12" s="31" t="s">
-        <v>174</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10" t="n">
-        <f aca="false">SUM(D5:D12)-D9</f>
-        <v>4453</v>
-      </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="10" t="n">
-        <f aca="false">SUM(G5:G10)</f>
-        <v>4129</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <f aca="false">G13-D13</f>
-        <v>-324</v>
-      </c>
-      <c r="I13" s="9"/>
+      <c r="G13" s="30" t="s">
+        <v>176</v>
+      </c>
+      <c r="H13" s="31" t="s">
+        <v>176</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="B14" s="32" t="n">
-        <v>0.23</v>
-      </c>
+        <v>184</v>
+      </c>
+      <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="10" t="n">
-        <f aca="false">D13*$B$14</f>
-        <v>1024.19</v>
+        <f aca="false">SUM(D5:D13)-D8</f>
+        <v>4145</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
       <c r="G14" s="10" t="n">
-        <f aca="false">G13*$B$14</f>
-        <v>949.67</v>
+        <f aca="false">SUM(G5:G11)</f>
+        <v>3865</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">G14-D14</f>
-        <v>-74.52</v>
+        <v>-280</v>
       </c>
       <c r="I14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="B15" s="9"/>
+        <v>185</v>
+      </c>
+      <c r="B15" s="32" t="n">
+        <v>0.23</v>
+      </c>
       <c r="C15" s="9"/>
       <c r="D15" s="10" t="n">
-        <f aca="false">D13+D14</f>
-        <v>5477.19</v>
+        <f aca="false">D14*$B$15</f>
+        <v>953.35</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
       <c r="G15" s="10" t="n">
-        <f aca="false">G13+G14</f>
-        <v>5078.67</v>
+        <f aca="false">G14*$B$15</f>
+        <v>888.95</v>
       </c>
       <c r="H15" s="10" t="n">
         <f aca="false">G15-D15</f>
-        <v>-398.52</v>
+        <v>-64.4</v>
       </c>
       <c r="I15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="A16" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="10" t="n">
+        <f aca="false">D14+D15</f>
+        <v>5098.35</v>
+      </c>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="10" t="n">
+        <f aca="false">G14+G15</f>
+        <v>4753.95</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <f aca="false">G16-D16</f>
+        <v>-344.400000000001</v>
+      </c>
+      <c r="I16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
-        <v>207</v>
-      </c>
+      <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -3854,7 +3888,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -3867,7 +3901,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3877,6 +3911,32 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3909,7 +3969,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3923,7 +3983,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3949,42 +4009,42 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C5" s="22" t="n">
         <v>3</v>
@@ -4008,18 +4068,18 @@
         <v>356.975609756098</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>16</v>
@@ -4043,18 +4103,18 @@
         <v>1359.86991869919</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C7" s="22" t="n">
         <v>12</v>
@@ -4078,18 +4138,18 @@
         <v>911.90243902439</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>1</v>
@@ -4116,15 +4176,15 @@
         <v>33</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="C9" s="22" t="n">
         <v>1</v>
@@ -4148,15 +4208,15 @@
         <v>61.2682926829268</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -4176,7 +4236,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -4192,12 +4252,12 @@
       </c>
       <c r="I11" s="9"/>
       <c r="J11" s="9" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -4213,12 +4273,12 @@
       </c>
       <c r="I12" s="9"/>
       <c r="J12" s="9" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -4238,7 +4298,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="34" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B14" s="34"/>
       <c r="C14" s="34"/>
@@ -4254,7 +4314,7 @@
       <c r="H14" s="34"/>
       <c r="I14" s="34"/>
       <c r="J14" s="34" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4271,7 +4331,7 @@
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="37" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B16" s="37"/>
       <c r="C16" s="37"/>
@@ -4285,7 +4345,7 @@
     </row>
     <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="37" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B17" s="37"/>
       <c r="C17" s="37"/>
@@ -4299,7 +4359,7 @@
     </row>
     <row r="18" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="37" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B18" s="37"/>
       <c r="C18" s="37"/>
@@ -4348,7 +4408,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4362,7 +4422,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4388,48 +4448,48 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">Necessidade!$C$29</f>
@@ -4437,7 +4497,7 @@
       </c>
       <c r="F5" s="39"/>
       <c r="G5" s="40" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="H5" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F5),IF(UPPER(G5)="S",F5/(1+$B$17),F5),"")</f>
@@ -4448,7 +4508,7 @@
         <v/>
       </c>
       <c r="J5" s="8" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4456,13 +4516,13 @@
         <v>33</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="E6" s="5" t="n">
         <f aca="false">Necessidade!$C$30</f>
@@ -4470,7 +4530,7 @@
       </c>
       <c r="F6" s="39"/>
       <c r="G6" s="40" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="H6" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F6),IF(UPPER(G6)="S",F6/(1+$B$17),F6),"")</f>
@@ -4481,28 +4541,28 @@
         <v/>
       </c>
       <c r="J6" s="8" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="39"/>
       <c r="G7" s="40" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="H7" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F7),IF(UPPER(G7)="S",F7/(1+$B$17),F7),"")</f>
@@ -4513,28 +4573,28 @@
         <v/>
       </c>
       <c r="J7" s="8" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="39"/>
       <c r="G8" s="40" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="H8" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F8),IF(UPPER(G8)="S",F8/(1+$B$17),F8),"")</f>
@@ -4545,21 +4605,21 @@
         <v/>
       </c>
       <c r="J8" s="8" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">Necessidade!$C$32</f>
@@ -4567,7 +4627,7 @@
       </c>
       <c r="F9" s="39"/>
       <c r="G9" s="40" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="H9" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F9),IF(UPPER(G9)="S",F9/(1+$B$17),F9),"")</f>
@@ -4578,21 +4638,21 @@
         <v/>
       </c>
       <c r="J9" s="8" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">Necessidade!$C$33</f>
@@ -4600,7 +4660,7 @@
       </c>
       <c r="F10" s="39"/>
       <c r="G10" s="40" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="H10" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F10),IF(UPPER(G10)="S",F10/(1+$B$17),F10),"")</f>
@@ -4611,21 +4671,21 @@
         <v/>
       </c>
       <c r="J10" s="8" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">Necessidade!$C$34</f>
@@ -4633,7 +4693,7 @@
       </c>
       <c r="F11" s="39"/>
       <c r="G11" s="40" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="H11" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F11),IF(UPPER(G11)="S",F11/(1+$B$17),F11),"")</f>
@@ -4644,18 +4704,18 @@
         <v/>
       </c>
       <c r="J11" s="8" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5" t="n">
@@ -4667,28 +4727,28 @@
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="8" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="39"/>
       <c r="G13" s="40" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="H13" s="6" t="str">
         <f aca="false">IF(ISNUMBER(F13),IF(UPPER(G13)="S",F13/(1+$B$17),F13),"")</f>
@@ -4699,12 +4759,12 @@
         <v/>
       </c>
       <c r="J13" s="8" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -4721,7 +4781,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -4738,7 +4798,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -4755,7 +4815,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="34" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="B17" s="35" t="n">
         <v>0.23</v>
@@ -4771,7 +4831,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="34" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B18" s="34"/>
       <c r="C18" s="34"/>
@@ -4800,7 +4860,7 @@
     </row>
     <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="37" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="B20" s="37"/>
       <c r="C20" s="37"/>
@@ -4814,7 +4874,7 @@
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="37" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B21" s="37"/>
       <c r="C21" s="37"/>
@@ -4828,7 +4888,7 @@
     </row>
     <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="37" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B22" s="37"/>
       <c r="C22" s="37"/>
@@ -4885,7 +4945,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4900,7 +4960,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4928,42 +4988,42 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">Necessidade!$C$29</f>
@@ -4985,11 +5045,11 @@
         <v>840</v>
       </c>
       <c r="G5" s="25" t="n">
-        <v>110</v>
+        <v>112.272727272727</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G5),$B5*G5,"")</f>
-        <v>1320</v>
+        <v>1347.27272727273</v>
       </c>
       <c r="I5" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$5),Vistaprint!$H$5,"")</f>
@@ -5000,7 +5060,7 @@
         <v/>
       </c>
       <c r="K5" s="8" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5026,12 +5086,10 @@
         <f aca="false">IF(ISNUMBER(E6),$B6*E6,"")</f>
         <v>222</v>
       </c>
-      <c r="G6" s="25" t="n">
-        <v>110</v>
-      </c>
-      <c r="H6" s="6" t="n">
+      <c r="G6" s="44"/>
+      <c r="H6" s="45" t="str">
         <f aca="false">IF(ISNUMBER(G6),$B6*G6,"")</f>
-        <v>330</v>
+        <v/>
       </c>
       <c r="I6" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$6),Vistaprint!$H$6,"")</f>
@@ -5042,31 +5100,33 @@
         <v/>
       </c>
       <c r="K6" s="8" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">Necessidade!$C$31</f>
         <v>4</v>
       </c>
-      <c r="C7" s="44"/>
+      <c r="C7" s="46"/>
       <c r="D7" s="45" t="str">
         <f aca="false">IF(ISNUMBER(C7),$B7*C7,"")</f>
         <v/>
       </c>
-      <c r="E7" s="46"/>
+      <c r="E7" s="44"/>
       <c r="F7" s="45" t="str">
         <f aca="false">IF(ISNUMBER(E7),$B7*E7,"")</f>
         <v/>
       </c>
-      <c r="G7" s="46"/>
-      <c r="H7" s="45" t="str">
+      <c r="G7" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="H7" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G7),$B7*G7,"")</f>
-        <v/>
+        <v>280</v>
       </c>
       <c r="I7" s="43" t="str">
         <f aca="false">IF(AND(ISNUMBER(Vistaprint!$H$7),ISNUMBER(Vistaprint!$H$8)),(Vistaprint!$I$7+Vistaprint!$I$8)/(Vistaprint!$E$7+Vistaprint!$E$8),"")</f>
@@ -5077,12 +5137,12 @@
         <v/>
       </c>
       <c r="K7" s="8" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">Necessidade!$C$32</f>
@@ -5104,11 +5164,11 @@
         <v>447</v>
       </c>
       <c r="G8" s="25" t="n">
-        <v>333</v>
+        <v>280</v>
       </c>
       <c r="H8" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G8),$B8*G8,"")</f>
-        <v>999</v>
+        <v>840</v>
       </c>
       <c r="I8" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$9),Vistaprint!$H$9,"")</f>
@@ -5119,12 +5179,12 @@
         <v/>
       </c>
       <c r="K8" s="8" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">Necessidade!$C$33</f>
@@ -5161,12 +5221,12 @@
         <v/>
       </c>
       <c r="K9" s="8" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Necessidade!$C$34</f>
@@ -5180,7 +5240,7 @@
         <f aca="false">IF(ISNUMBER(C10),$B10*C10,"")</f>
         <v>61.2682926829268</v>
       </c>
-      <c r="E10" s="46"/>
+      <c r="E10" s="44"/>
       <c r="F10" s="45" t="str">
         <f aca="false">IF(ISNUMBER(E10),$B10*E10,"")</f>
         <v/>
@@ -5201,44 +5261,44 @@
         <v/>
       </c>
       <c r="K10" s="8" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">Necessidade!$C$35</f>
         <v>1</v>
       </c>
-      <c r="C11" s="44"/>
+      <c r="C11" s="46"/>
       <c r="D11" s="45" t="str">
         <f aca="false">IF(ISNUMBER(C11),$B11*C11,"")</f>
         <v/>
       </c>
-      <c r="E11" s="46"/>
+      <c r="E11" s="44"/>
       <c r="F11" s="45" t="str">
         <f aca="false">IF(ISNUMBER(E11),$B11*E11,"")</f>
         <v/>
       </c>
-      <c r="G11" s="46"/>
+      <c r="G11" s="44"/>
       <c r="H11" s="45" t="str">
         <f aca="false">IF(ISNUMBER(G11),$B11*G11,"")</f>
         <v/>
       </c>
-      <c r="I11" s="44"/>
+      <c r="I11" s="46"/>
       <c r="J11" s="45" t="str">
         <f aca="false">IF(ISNUMBER(I11),$B11*I11,"")</f>
         <v/>
       </c>
       <c r="K11" s="8" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>1</v>
@@ -5258,10 +5318,12 @@
         <f aca="false">IF(ISNUMBER(E12),$B12*E12,"")</f>
         <v>15</v>
       </c>
-      <c r="G12" s="46"/>
-      <c r="H12" s="45" t="str">
+      <c r="G12" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="H12" s="6" t="n">
         <f aca="false">IF(ISNUMBER(G12),$B12*G12,"")</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="I12" s="43" t="str">
         <f aca="false">IF(ISNUMBER(Vistaprint!$H$13),Vistaprint!$H$13,"")</f>
@@ -5272,12 +5334,12 @@
         <v/>
       </c>
       <c r="K12" s="5" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>1</v>
@@ -5312,12 +5374,12 @@
         <v>0</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -5333,7 +5395,7 @@
       <c r="G14" s="9"/>
       <c r="H14" s="10" t="n">
         <f aca="false">SUM(H5:H13)</f>
-        <v>4129</v>
+        <v>3977.27272727273</v>
       </c>
       <c r="I14" s="9"/>
       <c r="J14" s="10" t="n">
@@ -5344,7 +5406,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B15" s="32" t="n">
         <v>0.23</v>
@@ -5362,7 +5424,7 @@
       <c r="G15" s="9"/>
       <c r="H15" s="10" t="n">
         <f aca="false">H14*$B$15</f>
-        <v>949.67</v>
+        <v>914.772727272727</v>
       </c>
       <c r="I15" s="9"/>
       <c r="J15" s="10" t="n">
@@ -5373,7 +5435,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -5389,7 +5451,7 @@
       <c r="G16" s="9"/>
       <c r="H16" s="10" t="n">
         <f aca="false">H14+H15</f>
-        <v>5078.67</v>
+        <v>4892.04545454546</v>
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="10" t="n">
@@ -5400,7 +5462,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="34" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B17" s="34"/>
       <c r="C17" s="34"/>
@@ -5416,7 +5478,7 @@
       <c r="G17" s="34"/>
       <c r="H17" s="34" t="n">
         <f aca="false">COUNTBLANK(G5:G13)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="34" t="n">
@@ -5427,7 +5489,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="34" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="B18" s="34"/>
       <c r="C18" s="34"/>
@@ -5440,7 +5502,7 @@
       <c r="G18" s="34"/>
       <c r="H18" s="47" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(($B$5:$B$12)*(G5:G12)*ISNUMBER($C$5:$C$12))/SUMPRODUCT(($B$5:$B$12)*($C$5:$C$12)*ISNUMBER(G5:G12)),"")</f>
-        <v>1.47744846528467</v>
+        <v>1.37444251993081</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="47" t="str">
@@ -5464,7 +5526,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -5479,7 +5541,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -5494,7 +5556,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -5509,7 +5571,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>

</xml_diff>